<commit_message>
Restore كشف الحساب sheet in workbook
</commit_message>
<xml_diff>
--- a/output/lead6_report.xlsx
+++ b/output/lead6_report.xlsx
@@ -10,9 +10,11 @@
     <sheet name="تفاصيل شهر 6" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="الاسعار" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="العمليات المالية" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="كشف الحساب" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'تفاصيل شهر 6'!$A$1:$X$332</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'كشف الحساب'!$A$9:$C$13</definedName>
   </definedNames>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,16 +22,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="[$-2000401]0"/>
     <numFmt numFmtId="165" formatCode="[$-2000401]0.#"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="167" formatCode="#,##0.00 &quot;ريال&quot;"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="168" formatCode="0.00 &quot;كجم&quot;"/>
     <numFmt numFmtId="169" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="170" formatCode="0.00 &quot;كجم&quot;"/>
+    <numFmt numFmtId="170" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="171" formatCode="#,##0.00 &quot;SAR&quot;"/>
+    <numFmt numFmtId="172" formatCode="yyyy/mm/dd"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="28">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -165,8 +169,29 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007C6B68"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="005B4A47"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002F2628"/>
+    </font>
+    <font>
+      <color rgb="002A2425"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -209,8 +234,28 @@
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B4A47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F2628"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F1EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF1F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -312,11 +357,25 @@
         <color rgb="00D9E2EC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E1D4CA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E1D4CA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E1D4CA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E1D4CA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -403,7 +462,7 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -452,8 +511,47 @@
     <xf numFmtId="0" fontId="20" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="26" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="27" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="27" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -871,13 +969,6 @@
           <t>2026-06-01 - 2026-06-13</t>
         </is>
       </c>
-      <c r="B1" s="34" t="n"/>
-      <c r="C1" s="34" t="n"/>
-      <c r="D1" s="34" t="n"/>
-      <c r="E1" s="34" t="n"/>
-      <c r="F1" s="34" t="n"/>
-      <c r="G1" s="34" t="n"/>
-      <c r="H1" s="34" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="34" t="n"/>
@@ -1946,7 +2037,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L2" s="42" t="n">
+      <c r="L2" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M2" s="40" t="inlineStr">
@@ -2038,7 +2129,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L3" s="42" t="n">
+      <c r="L3" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M3" s="40" t="inlineStr">
@@ -2130,7 +2221,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L4" s="42" t="n">
+      <c r="L4" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M4" s="40" t="inlineStr">
@@ -2222,7 +2313,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L5" s="42" t="n">
+      <c r="L5" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M5" s="40" t="inlineStr">
@@ -2314,7 +2405,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L6" s="42" t="n">
+      <c r="L6" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M6" s="40" t="inlineStr">
@@ -2406,7 +2497,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L7" s="42" t="n">
+      <c r="L7" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M7" s="40" t="inlineStr">
@@ -2498,7 +2589,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L8" s="42" t="n">
+      <c r="L8" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M8" s="40" t="inlineStr">
@@ -2590,7 +2681,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L9" s="42" t="n">
+      <c r="L9" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M9" s="40" t="inlineStr">
@@ -2682,7 +2773,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L10" s="42" t="n">
+      <c r="L10" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M10" s="40" t="inlineStr">
@@ -2774,7 +2865,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L11" s="42" t="n">
+      <c r="L11" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M11" s="40" t="inlineStr">
@@ -2866,7 +2957,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L12" s="42" t="n">
+      <c r="L12" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
@@ -2958,7 +3049,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L13" s="42" t="n">
+      <c r="L13" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M13" s="40" t="inlineStr">
@@ -3050,7 +3141,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L14" s="42" t="n">
+      <c r="L14" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M14" s="40" t="inlineStr">
@@ -3142,7 +3233,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L15" s="42" t="n">
+      <c r="L15" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M15" s="40" t="inlineStr">
@@ -3234,7 +3325,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L16" s="42" t="n">
+      <c r="L16" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M16" s="40" t="inlineStr">
@@ -3326,7 +3417,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L17" s="42" t="n">
+      <c r="L17" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M17" s="40" t="inlineStr">
@@ -3418,7 +3509,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L18" s="42" t="n">
+      <c r="L18" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M18" s="40" t="inlineStr">
@@ -3510,7 +3601,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L19" s="42" t="n">
+      <c r="L19" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M19" s="40" t="inlineStr">
@@ -3602,7 +3693,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L20" s="42" t="n">
+      <c r="L20" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M20" s="40" t="inlineStr">
@@ -3694,7 +3785,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L21" s="42" t="n">
+      <c r="L21" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M21" s="40" t="inlineStr">
@@ -3786,7 +3877,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L22" s="42" t="n">
+      <c r="L22" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M22" s="40" t="inlineStr">
@@ -3878,7 +3969,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L23" s="42" t="n">
+      <c r="L23" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M23" s="40" t="inlineStr">
@@ -3970,7 +4061,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L24" s="42" t="n">
+      <c r="L24" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M24" s="40" t="inlineStr">
@@ -4062,7 +4153,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L25" s="42" t="n">
+      <c r="L25" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M25" s="40" t="inlineStr">
@@ -4154,7 +4245,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L26" s="42" t="n">
+      <c r="L26" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M26" s="40" t="inlineStr">
@@ -4246,7 +4337,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L27" s="42" t="n">
+      <c r="L27" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M27" s="40" t="inlineStr">
@@ -4338,7 +4429,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L28" s="42" t="n">
+      <c r="L28" s="60" t="n">
         <v>3</v>
       </c>
       <c r="M28" s="40" t="inlineStr">
@@ -4430,7 +4521,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L29" s="42" t="n">
+      <c r="L29" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M29" s="40" t="inlineStr">
@@ -4522,7 +4613,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L30" s="42" t="n">
+      <c r="L30" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M30" s="40" t="inlineStr">
@@ -4614,7 +4705,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L31" s="42" t="n">
+      <c r="L31" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M31" s="40" t="inlineStr">
@@ -4706,7 +4797,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L32" s="42" t="n">
+      <c r="L32" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M32" s="40" t="inlineStr">
@@ -4798,7 +4889,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L33" s="42" t="n">
+      <c r="L33" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M33" s="40" t="inlineStr">
@@ -4890,7 +4981,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L34" s="42" t="n">
+      <c r="L34" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M34" s="40" t="inlineStr">
@@ -4982,7 +5073,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L35" s="42" t="n">
+      <c r="L35" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M35" s="40" t="inlineStr">
@@ -5074,7 +5165,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L36" s="42" t="n">
+      <c r="L36" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M36" s="40" t="inlineStr">
@@ -5166,7 +5257,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L37" s="42" t="n">
+      <c r="L37" s="60" t="n">
         <v>3</v>
       </c>
       <c r="M37" s="40" t="inlineStr">
@@ -5258,7 +5349,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L38" s="42" t="n">
+      <c r="L38" s="60" t="n">
         <v>15</v>
       </c>
       <c r="M38" s="40" t="inlineStr">
@@ -5352,7 +5443,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="L39" s="42" t="n">
+      <c r="L39" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M39" s="40" t="inlineStr">
@@ -5444,7 +5535,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L40" s="42" t="n">
+      <c r="L40" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M40" s="40" t="inlineStr">
@@ -5536,7 +5627,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L41" s="42" t="n">
+      <c r="L41" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M41" s="40" t="inlineStr">
@@ -5628,7 +5719,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L42" s="42" t="n">
+      <c r="L42" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M42" s="40" t="inlineStr">
@@ -5720,7 +5811,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L43" s="42" t="n">
+      <c r="L43" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M43" s="40" t="inlineStr">
@@ -5812,7 +5903,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L44" s="42" t="n">
+      <c r="L44" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M44" s="40" t="inlineStr">
@@ -5904,7 +5995,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L45" s="42" t="n">
+      <c r="L45" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M45" s="40" t="inlineStr">
@@ -5996,7 +6087,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L46" s="42" t="n">
+      <c r="L46" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M46" s="40" t="inlineStr">
@@ -6088,7 +6179,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L47" s="42" t="n">
+      <c r="L47" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M47" s="40" t="inlineStr">
@@ -6180,7 +6271,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L48" s="42" t="n">
+      <c r="L48" s="60" t="n">
         <v>15</v>
       </c>
       <c r="M48" s="40" t="inlineStr">
@@ -6272,7 +6363,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L49" s="42" t="n">
+      <c r="L49" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M49" s="40" t="inlineStr">
@@ -6364,7 +6455,7 @@
           <t>ارامكس - ARAMEX</t>
         </is>
       </c>
-      <c r="L50" s="42" t="n">
+      <c r="L50" s="60" t="n">
         <v>10</v>
       </c>
       <c r="M50" s="40" t="inlineStr">
@@ -6456,7 +6547,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L51" s="42" t="n">
+      <c r="L51" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M51" s="40" t="inlineStr">
@@ -6548,7 +6639,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L52" s="42" t="n">
+      <c r="L52" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M52" s="40" t="inlineStr">
@@ -6640,7 +6731,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L53" s="42" t="n">
+      <c r="L53" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M53" s="40" t="inlineStr">
@@ -6732,7 +6823,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L54" s="42" t="n">
+      <c r="L54" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M54" s="40" t="inlineStr">
@@ -6824,7 +6915,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L55" s="42" t="n">
+      <c r="L55" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M55" s="40" t="inlineStr">
@@ -6916,7 +7007,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L56" s="42" t="n">
+      <c r="L56" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M56" s="40" t="inlineStr">
@@ -7008,7 +7099,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L57" s="42" t="n">
+      <c r="L57" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M57" s="40" t="inlineStr">
@@ -7100,7 +7191,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L58" s="42" t="n">
+      <c r="L58" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M58" s="40" t="inlineStr">
@@ -7192,7 +7283,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L59" s="42" t="n">
+      <c r="L59" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M59" s="40" t="inlineStr">
@@ -7284,7 +7375,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L60" s="42" t="n">
+      <c r="L60" s="60" t="n">
         <v>4</v>
       </c>
       <c r="M60" s="40" t="inlineStr">
@@ -7376,7 +7467,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L61" s="42" t="n">
+      <c r="L61" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M61" s="40" t="inlineStr">
@@ -7468,7 +7559,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L62" s="42" t="n">
+      <c r="L62" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M62" s="40" t="inlineStr">
@@ -7560,7 +7651,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L63" s="42" t="n">
+      <c r="L63" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M63" s="40" t="inlineStr">
@@ -7652,7 +7743,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L64" s="42" t="n">
+      <c r="L64" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M64" s="40" t="inlineStr">
@@ -7744,7 +7835,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L65" s="42" t="n">
+      <c r="L65" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M65" s="40" t="inlineStr">
@@ -7836,7 +7927,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L66" s="42" t="n">
+      <c r="L66" s="60" t="n">
         <v>10</v>
       </c>
       <c r="M66" s="40" t="inlineStr">
@@ -7928,7 +8019,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L67" s="42" t="n">
+      <c r="L67" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M67" s="40" t="inlineStr">
@@ -8020,7 +8111,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L68" s="42" t="n">
+      <c r="L68" s="60" t="n">
         <v>3</v>
       </c>
       <c r="M68" s="40" t="inlineStr">
@@ -8112,7 +8203,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L69" s="42" t="n">
+      <c r="L69" s="60" t="n">
         <v>4</v>
       </c>
       <c r="M69" s="40" t="inlineStr">
@@ -8204,7 +8295,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L70" s="42" t="n">
+      <c r="L70" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M70" s="40" t="inlineStr">
@@ -8296,7 +8387,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L71" s="42" t="n">
+      <c r="L71" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M71" s="40" t="inlineStr">
@@ -8388,7 +8479,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L72" s="42" t="n">
+      <c r="L72" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M72" s="40" t="inlineStr">
@@ -8480,7 +8571,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L73" s="42" t="n">
+      <c r="L73" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M73" s="40" t="inlineStr">
@@ -8572,7 +8663,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L74" s="42" t="n">
+      <c r="L74" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M74" s="40" t="inlineStr">
@@ -8664,7 +8755,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L75" s="42" t="n">
+      <c r="L75" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M75" s="40" t="inlineStr">
@@ -8756,7 +8847,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L76" s="42" t="n">
+      <c r="L76" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M76" s="40" t="inlineStr">
@@ -8848,7 +8939,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L77" s="42" t="n">
+      <c r="L77" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M77" s="40" t="inlineStr">
@@ -8940,7 +9031,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L78" s="42" t="n">
+      <c r="L78" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M78" s="40" t="inlineStr">
@@ -9032,7 +9123,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L79" s="42" t="n">
+      <c r="L79" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M79" s="40" t="inlineStr">
@@ -9124,7 +9215,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L80" s="42" t="n">
+      <c r="L80" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M80" s="40" t="inlineStr">
@@ -9216,7 +9307,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L81" s="42" t="n">
+      <c r="L81" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M81" s="40" t="inlineStr">
@@ -9308,7 +9399,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L82" s="42" t="n">
+      <c r="L82" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M82" s="40" t="inlineStr">
@@ -9400,7 +9491,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L83" s="42" t="n">
+      <c r="L83" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M83" s="40" t="inlineStr">
@@ -9492,7 +9583,7 @@
           <t>ارامكس - ARAMEX</t>
         </is>
       </c>
-      <c r="L84" s="42" t="n">
+      <c r="L84" s="60" t="n">
         <v>20</v>
       </c>
       <c r="M84" s="40" t="inlineStr">
@@ -9584,7 +9675,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L85" s="42" t="n">
+      <c r="L85" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M85" s="40" t="inlineStr">
@@ -9676,7 +9767,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L86" s="42" t="n">
+      <c r="L86" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M86" s="40" t="inlineStr">
@@ -9768,7 +9859,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L87" s="42" t="n">
+      <c r="L87" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M87" s="40" t="inlineStr">
@@ -9860,7 +9951,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L88" s="42" t="n">
+      <c r="L88" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M88" s="40" t="inlineStr">
@@ -9952,7 +10043,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L89" s="42" t="n">
+      <c r="L89" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M89" s="40" t="inlineStr">
@@ -10044,7 +10135,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L90" s="42" t="n">
+      <c r="L90" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M90" s="40" t="inlineStr">
@@ -10136,7 +10227,7 @@
           <t>ارامكس - ARAMEX</t>
         </is>
       </c>
-      <c r="L91" s="42" t="n">
+      <c r="L91" s="60" t="n">
         <v>0.85</v>
       </c>
       <c r="M91" s="40" t="inlineStr">
@@ -10228,7 +10319,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L92" s="42" t="n">
+      <c r="L92" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M92" s="40" t="inlineStr">
@@ -10320,7 +10411,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L93" s="42" t="n">
+      <c r="L93" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M93" s="40" t="inlineStr">
@@ -10412,7 +10503,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L94" s="42" t="n">
+      <c r="L94" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M94" s="40" t="inlineStr">
@@ -10504,7 +10595,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L95" s="42" t="n">
+      <c r="L95" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M95" s="40" t="inlineStr">
@@ -10596,7 +10687,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L96" s="42" t="n">
+      <c r="L96" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M96" s="40" t="inlineStr">
@@ -10688,7 +10779,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L97" s="42" t="n">
+      <c r="L97" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M97" s="40" t="inlineStr">
@@ -10780,7 +10871,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L98" s="42" t="n">
+      <c r="L98" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M98" s="40" t="inlineStr">
@@ -10872,7 +10963,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L99" s="42" t="n">
+      <c r="L99" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M99" s="40" t="inlineStr">
@@ -10964,7 +11055,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L100" s="42" t="n">
+      <c r="L100" s="60" t="n">
         <v>3</v>
       </c>
       <c r="M100" s="40" t="inlineStr">
@@ -11056,7 +11147,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L101" s="42" t="n">
+      <c r="L101" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M101" s="40" t="inlineStr">
@@ -11148,7 +11239,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L102" s="42" t="n">
+      <c r="L102" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M102" s="40" t="inlineStr">
@@ -11240,7 +11331,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L103" s="42" t="n">
+      <c r="L103" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M103" s="40" t="inlineStr">
@@ -11332,7 +11423,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L104" s="42" t="n">
+      <c r="L104" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M104" s="40" t="inlineStr">
@@ -11424,7 +11515,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L105" s="42" t="n">
+      <c r="L105" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M105" s="40" t="inlineStr">
@@ -11516,7 +11607,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L106" s="42" t="n">
+      <c r="L106" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M106" s="40" t="inlineStr">
@@ -11608,7 +11699,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L107" s="42" t="n">
+      <c r="L107" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M107" s="40" t="inlineStr">
@@ -11700,7 +11791,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L108" s="42" t="n">
+      <c r="L108" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M108" s="40" t="inlineStr">
@@ -11792,7 +11883,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L109" s="42" t="n">
+      <c r="L109" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M109" s="40" t="inlineStr">
@@ -11884,7 +11975,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L110" s="42" t="n">
+      <c r="L110" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M110" s="40" t="inlineStr">
@@ -11976,7 +12067,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L111" s="42" t="n">
+      <c r="L111" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M111" s="40" t="inlineStr">
@@ -12068,7 +12159,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L112" s="42" t="n">
+      <c r="L112" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M112" s="40" t="inlineStr">
@@ -12160,7 +12251,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L113" s="42" t="n">
+      <c r="L113" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M113" s="40" t="inlineStr">
@@ -12252,7 +12343,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L114" s="42" t="n">
+      <c r="L114" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M114" s="40" t="inlineStr">
@@ -12344,7 +12435,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L115" s="42" t="n">
+      <c r="L115" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M115" s="40" t="inlineStr">
@@ -12436,7 +12527,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L116" s="42" t="n">
+      <c r="L116" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M116" s="40" t="inlineStr">
@@ -12528,7 +12619,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L117" s="42" t="n">
+      <c r="L117" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M117" s="40" t="inlineStr">
@@ -12620,7 +12711,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L118" s="42" t="n">
+      <c r="L118" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M118" s="40" t="inlineStr">
@@ -12712,7 +12803,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L119" s="42" t="n">
+      <c r="L119" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M119" s="40" t="inlineStr">
@@ -12804,7 +12895,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L120" s="42" t="n">
+      <c r="L120" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M120" s="40" t="inlineStr">
@@ -12896,7 +12987,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L121" s="42" t="n">
+      <c r="L121" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M121" s="40" t="inlineStr">
@@ -12988,7 +13079,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L122" s="42" t="n">
+      <c r="L122" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M122" s="40" t="inlineStr">
@@ -13080,7 +13171,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L123" s="42" t="n">
+      <c r="L123" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M123" s="40" t="inlineStr">
@@ -13172,7 +13263,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L124" s="42" t="n">
+      <c r="L124" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M124" s="40" t="inlineStr">
@@ -13264,7 +13355,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L125" s="42" t="n">
+      <c r="L125" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M125" s="40" t="inlineStr">
@@ -13356,7 +13447,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L126" s="42" t="n">
+      <c r="L126" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M126" s="40" t="inlineStr">
@@ -13448,7 +13539,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L127" s="42" t="n">
+      <c r="L127" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M127" s="40" t="inlineStr">
@@ -13540,7 +13631,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L128" s="42" t="n">
+      <c r="L128" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M128" s="40" t="inlineStr">
@@ -13632,7 +13723,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L129" s="42" t="n">
+      <c r="L129" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M129" s="40" t="inlineStr">
@@ -13724,7 +13815,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L130" s="42" t="n">
+      <c r="L130" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M130" s="40" t="inlineStr">
@@ -13816,7 +13907,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L131" s="42" t="n">
+      <c r="L131" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M131" s="40" t="inlineStr">
@@ -13908,7 +13999,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L132" s="42" t="n">
+      <c r="L132" s="60" t="n">
         <v>4</v>
       </c>
       <c r="M132" s="40" t="inlineStr">
@@ -14000,7 +14091,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L133" s="42" t="n">
+      <c r="L133" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M133" s="40" t="inlineStr">
@@ -14092,7 +14183,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L134" s="42" t="n">
+      <c r="L134" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M134" s="40" t="inlineStr">
@@ -14184,7 +14275,7 @@
           <t>ارامكس - ARAMEX</t>
         </is>
       </c>
-      <c r="L135" s="42" t="n">
+      <c r="L135" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M135" s="40" t="inlineStr">
@@ -14276,7 +14367,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L136" s="42" t="n">
+      <c r="L136" s="60" t="n">
         <v>15</v>
       </c>
       <c r="M136" s="40" t="inlineStr">
@@ -14368,7 +14459,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L137" s="42" t="n">
+      <c r="L137" s="60" t="n">
         <v>10</v>
       </c>
       <c r="M137" s="40" t="inlineStr">
@@ -14460,7 +14551,7 @@
           <t>SMSA ( استلام من الفرع )</t>
         </is>
       </c>
-      <c r="L138" s="42" t="n">
+      <c r="L138" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M138" s="40" t="inlineStr">
@@ -14552,7 +14643,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L139" s="42" t="n">
+      <c r="L139" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M139" s="40" t="inlineStr">
@@ -14644,7 +14735,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L140" s="42" t="n">
+      <c r="L140" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M140" s="40" t="inlineStr">
@@ -14736,7 +14827,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L141" s="42" t="n">
+      <c r="L141" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M141" s="40" t="inlineStr">
@@ -14828,7 +14919,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L142" s="42" t="n">
+      <c r="L142" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M142" s="40" t="inlineStr">
@@ -14920,7 +15011,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L143" s="42" t="n">
+      <c r="L143" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M143" s="40" t="inlineStr">
@@ -15012,7 +15103,7 @@
           <t>ارامكس - ARAMEX</t>
         </is>
       </c>
-      <c r="L144" s="42" t="n">
+      <c r="L144" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M144" s="40" t="inlineStr">
@@ -15104,7 +15195,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L145" s="42" t="n">
+      <c r="L145" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M145" s="40" t="inlineStr">
@@ -15196,7 +15287,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L146" s="42" t="n">
+      <c r="L146" s="60" t="n">
         <v>3</v>
       </c>
       <c r="M146" s="40" t="inlineStr">
@@ -15288,7 +15379,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L147" s="42" t="n">
+      <c r="L147" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M147" s="40" t="inlineStr">
@@ -15380,7 +15471,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L148" s="42" t="n">
+      <c r="L148" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M148" s="40" t="inlineStr">
@@ -15472,7 +15563,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L149" s="42" t="n">
+      <c r="L149" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M149" s="40" t="inlineStr">
@@ -15564,7 +15655,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L150" s="42" t="n">
+      <c r="L150" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M150" s="40" t="inlineStr">
@@ -15656,7 +15747,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L151" s="42" t="n">
+      <c r="L151" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M151" s="40" t="inlineStr">
@@ -15748,7 +15839,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L152" s="42" t="n">
+      <c r="L152" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M152" s="40" t="inlineStr">
@@ -15840,7 +15931,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L153" s="42" t="n">
+      <c r="L153" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M153" s="40" t="inlineStr">
@@ -15932,7 +16023,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L154" s="42" t="n">
+      <c r="L154" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M154" s="40" t="inlineStr">
@@ -16024,7 +16115,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L155" s="42" t="n">
+      <c r="L155" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M155" s="40" t="inlineStr">
@@ -16116,7 +16207,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L156" s="42" t="n">
+      <c r="L156" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M156" s="40" t="inlineStr">
@@ -16208,7 +16299,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L157" s="42" t="n">
+      <c r="L157" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M157" s="40" t="inlineStr">
@@ -16300,7 +16391,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L158" s="42" t="n">
+      <c r="L158" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M158" s="40" t="inlineStr">
@@ -16392,7 +16483,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L159" s="42" t="n">
+      <c r="L159" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M159" s="40" t="inlineStr">
@@ -16484,7 +16575,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L160" s="42" t="n">
+      <c r="L160" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M160" s="40" t="inlineStr">
@@ -16576,7 +16667,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L161" s="42" t="n">
+      <c r="L161" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M161" s="40" t="inlineStr">
@@ -16668,7 +16759,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L162" s="42" t="n">
+      <c r="L162" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M162" s="40" t="inlineStr">
@@ -16760,7 +16851,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L163" s="42" t="n">
+      <c r="L163" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M163" s="40" t="inlineStr">
@@ -16852,7 +16943,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L164" s="42" t="n">
+      <c r="L164" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M164" s="40" t="inlineStr">
@@ -16944,7 +17035,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L165" s="42" t="n">
+      <c r="L165" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M165" s="40" t="inlineStr">
@@ -17036,7 +17127,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L166" s="42" t="n">
+      <c r="L166" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M166" s="40" t="inlineStr">
@@ -17128,7 +17219,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L167" s="42" t="n">
+      <c r="L167" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M167" s="40" t="inlineStr">
@@ -17220,7 +17311,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L168" s="42" t="n">
+      <c r="L168" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M168" s="40" t="inlineStr">
@@ -17312,7 +17403,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L169" s="42" t="n">
+      <c r="L169" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M169" s="40" t="inlineStr">
@@ -17404,7 +17495,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L170" s="42" t="n">
+      <c r="L170" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M170" s="40" t="inlineStr">
@@ -17496,7 +17587,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L171" s="42" t="n">
+      <c r="L171" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M171" s="40" t="inlineStr">
@@ -17588,7 +17679,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L172" s="42" t="n">
+      <c r="L172" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M172" s="40" t="inlineStr">
@@ -17680,7 +17771,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L173" s="42" t="n">
+      <c r="L173" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M173" s="40" t="inlineStr">
@@ -17772,7 +17863,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L174" s="42" t="n">
+      <c r="L174" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M174" s="40" t="inlineStr">
@@ -17864,7 +17955,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L175" s="42" t="n">
+      <c r="L175" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M175" s="40" t="inlineStr">
@@ -17956,7 +18047,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L176" s="42" t="n">
+      <c r="L176" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M176" s="40" t="inlineStr">
@@ -18048,7 +18139,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L177" s="42" t="n">
+      <c r="L177" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M177" s="40" t="inlineStr">
@@ -18140,7 +18231,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L178" s="42" t="n">
+      <c r="L178" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M178" s="40" t="inlineStr">
@@ -18232,7 +18323,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L179" s="42" t="n">
+      <c r="L179" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M179" s="40" t="inlineStr">
@@ -18324,7 +18415,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L180" s="42" t="n">
+      <c r="L180" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M180" s="40" t="inlineStr">
@@ -18416,7 +18507,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L181" s="42" t="n">
+      <c r="L181" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M181" s="40" t="inlineStr">
@@ -18508,7 +18599,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L182" s="42" t="n">
+      <c r="L182" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M182" s="40" t="inlineStr">
@@ -18600,7 +18691,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L183" s="42" t="n">
+      <c r="L183" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M183" s="40" t="inlineStr">
@@ -18692,7 +18783,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L184" s="42" t="n">
+      <c r="L184" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M184" s="40" t="inlineStr">
@@ -18784,7 +18875,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L185" s="42" t="n">
+      <c r="L185" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M185" s="40" t="inlineStr">
@@ -18876,7 +18967,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L186" s="42" t="n">
+      <c r="L186" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M186" s="40" t="inlineStr">
@@ -18968,7 +19059,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L187" s="42" t="n">
+      <c r="L187" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M187" s="40" t="inlineStr">
@@ -19060,7 +19151,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L188" s="42" t="n">
+      <c r="L188" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M188" s="40" t="inlineStr">
@@ -19152,7 +19243,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L189" s="42" t="n">
+      <c r="L189" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M189" s="40" t="inlineStr">
@@ -19244,7 +19335,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L190" s="42" t="n">
+      <c r="L190" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M190" s="40" t="inlineStr">
@@ -19336,7 +19427,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L191" s="42" t="n">
+      <c r="L191" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M191" s="40" t="inlineStr">
@@ -19428,7 +19519,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L192" s="42" t="n">
+      <c r="L192" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M192" s="40" t="inlineStr">
@@ -19520,7 +19611,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L193" s="42" t="n">
+      <c r="L193" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M193" s="40" t="inlineStr">
@@ -19612,7 +19703,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L194" s="42" t="n">
+      <c r="L194" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M194" s="40" t="inlineStr">
@@ -19704,7 +19795,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L195" s="42" t="n">
+      <c r="L195" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M195" s="40" t="inlineStr">
@@ -19796,7 +19887,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L196" s="42" t="n">
+      <c r="L196" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M196" s="40" t="inlineStr">
@@ -19888,7 +19979,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L197" s="42" t="n">
+      <c r="L197" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M197" s="40" t="inlineStr">
@@ -19980,7 +20071,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L198" s="42" t="n">
+      <c r="L198" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M198" s="40" t="inlineStr">
@@ -20072,7 +20163,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L199" s="42" t="n">
+      <c r="L199" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M199" s="40" t="inlineStr">
@@ -20164,7 +20255,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L200" s="42" t="n">
+      <c r="L200" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M200" s="40" t="inlineStr">
@@ -20256,7 +20347,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L201" s="42" t="n">
+      <c r="L201" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M201" s="40" t="inlineStr">
@@ -20348,7 +20439,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L202" s="42" t="n">
+      <c r="L202" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M202" s="40" t="inlineStr">
@@ -20440,7 +20531,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L203" s="42" t="n">
+      <c r="L203" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M203" s="40" t="inlineStr">
@@ -20532,7 +20623,7 @@
           <t>RedBox - ريدبوكس</t>
         </is>
       </c>
-      <c r="L204" s="42" t="n">
+      <c r="L204" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M204" s="40" t="inlineStr">
@@ -20624,7 +20715,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L205" s="42" t="n">
+      <c r="L205" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M205" s="40" t="inlineStr">
@@ -20716,7 +20807,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L206" s="42" t="n">
+      <c r="L206" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M206" s="40" t="inlineStr">
@@ -20808,7 +20899,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L207" s="42" t="n">
+      <c r="L207" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M207" s="40" t="inlineStr">
@@ -20902,7 +20993,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="L208" s="42" t="n">
+      <c r="L208" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M208" s="40" t="inlineStr">
@@ -20996,7 +21087,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="L209" s="42" t="n">
+      <c r="L209" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M209" s="40" t="inlineStr">
@@ -21088,7 +21179,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L210" s="42" t="n">
+      <c r="L210" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M210" s="40" t="inlineStr">
@@ -21180,7 +21271,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L211" s="42" t="n">
+      <c r="L211" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M211" s="40" t="inlineStr">
@@ -21272,7 +21363,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L212" s="42" t="n">
+      <c r="L212" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M212" s="40" t="inlineStr">
@@ -21364,7 +21455,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L213" s="42" t="n">
+      <c r="L213" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M213" s="40" t="inlineStr">
@@ -21456,7 +21547,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L214" s="42" t="n">
+      <c r="L214" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M214" s="40" t="inlineStr">
@@ -21548,7 +21639,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L215" s="42" t="n">
+      <c r="L215" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M215" s="40" t="inlineStr">
@@ -21640,7 +21731,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L216" s="42" t="n">
+      <c r="L216" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M216" s="40" t="inlineStr">
@@ -21732,7 +21823,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L217" s="42" t="n">
+      <c r="L217" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M217" s="40" t="inlineStr">
@@ -21824,7 +21915,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L218" s="42" t="n">
+      <c r="L218" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M218" s="40" t="inlineStr">
@@ -21916,7 +22007,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L219" s="42" t="n">
+      <c r="L219" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M219" s="40" t="inlineStr">
@@ -22008,7 +22099,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L220" s="42" t="n">
+      <c r="L220" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M220" s="40" t="inlineStr">
@@ -22100,7 +22191,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L221" s="42" t="n">
+      <c r="L221" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M221" s="40" t="inlineStr">
@@ -22192,7 +22283,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L222" s="42" t="n">
+      <c r="L222" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M222" s="40" t="inlineStr">
@@ -22284,7 +22375,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L223" s="42" t="n">
+      <c r="L223" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M223" s="40" t="inlineStr">
@@ -22376,7 +22467,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L224" s="42" t="n">
+      <c r="L224" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M224" s="40" t="inlineStr">
@@ -22468,7 +22559,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L225" s="42" t="n">
+      <c r="L225" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M225" s="40" t="inlineStr">
@@ -22560,7 +22651,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L226" s="42" t="n">
+      <c r="L226" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M226" s="40" t="inlineStr">
@@ -22652,7 +22743,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L227" s="42" t="n">
+      <c r="L227" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M227" s="40" t="inlineStr">
@@ -22744,7 +22835,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L228" s="42" t="n">
+      <c r="L228" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M228" s="40" t="inlineStr">
@@ -22836,7 +22927,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L229" s="42" t="n">
+      <c r="L229" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M229" s="40" t="inlineStr">
@@ -22928,7 +23019,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L230" s="42" t="n">
+      <c r="L230" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M230" s="40" t="inlineStr">
@@ -23020,7 +23111,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L231" s="42" t="n">
+      <c r="L231" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M231" s="40" t="inlineStr">
@@ -23112,7 +23203,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L232" s="42" t="n">
+      <c r="L232" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M232" s="40" t="inlineStr">
@@ -23204,7 +23295,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L233" s="42" t="n">
+      <c r="L233" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M233" s="40" t="inlineStr">
@@ -23296,7 +23387,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L234" s="42" t="n">
+      <c r="L234" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M234" s="40" t="inlineStr">
@@ -23388,7 +23479,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L235" s="42" t="n">
+      <c r="L235" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M235" s="40" t="inlineStr">
@@ -23480,7 +23571,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L236" s="42" t="n">
+      <c r="L236" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M236" s="40" t="inlineStr">
@@ -23572,7 +23663,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L237" s="42" t="n">
+      <c r="L237" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M237" s="40" t="inlineStr">
@@ -23664,7 +23755,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L238" s="42" t="n">
+      <c r="L238" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M238" s="40" t="inlineStr">
@@ -23756,7 +23847,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L239" s="42" t="n">
+      <c r="L239" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M239" s="40" t="inlineStr">
@@ -23848,7 +23939,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L240" s="42" t="n">
+      <c r="L240" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M240" s="40" t="inlineStr">
@@ -23940,7 +24031,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L241" s="42" t="n">
+      <c r="L241" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M241" s="40" t="inlineStr">
@@ -24032,7 +24123,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L242" s="42" t="n">
+      <c r="L242" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M242" s="40" t="inlineStr">
@@ -24124,7 +24215,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L243" s="42" t="n">
+      <c r="L243" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M243" s="40" t="inlineStr">
@@ -24216,7 +24307,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L244" s="42" t="n">
+      <c r="L244" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M244" s="40" t="inlineStr">
@@ -24308,7 +24399,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L245" s="42" t="n">
+      <c r="L245" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M245" s="40" t="inlineStr">
@@ -24400,7 +24491,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L246" s="42" t="n">
+      <c r="L246" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M246" s="40" t="inlineStr">
@@ -24492,7 +24583,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L247" s="42" t="n">
+      <c r="L247" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M247" s="40" t="inlineStr">
@@ -24584,7 +24675,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L248" s="42" t="n">
+      <c r="L248" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M248" s="40" t="inlineStr">
@@ -24676,7 +24767,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L249" s="42" t="n">
+      <c r="L249" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M249" s="40" t="inlineStr">
@@ -24768,7 +24859,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L250" s="42" t="n">
+      <c r="L250" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M250" s="40" t="inlineStr">
@@ -24860,7 +24951,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L251" s="42" t="n">
+      <c r="L251" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M251" s="40" t="inlineStr">
@@ -24952,7 +25043,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L252" s="42" t="n">
+      <c r="L252" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M252" s="40" t="inlineStr">
@@ -25044,7 +25135,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L253" s="42" t="n">
+      <c r="L253" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M253" s="40" t="inlineStr">
@@ -25136,7 +25227,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L254" s="42" t="n">
+      <c r="L254" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M254" s="40" t="inlineStr">
@@ -25228,7 +25319,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L255" s="42" t="n">
+      <c r="L255" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M255" s="40" t="inlineStr">
@@ -25320,7 +25411,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L256" s="42" t="n">
+      <c r="L256" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M256" s="40" t="inlineStr">
@@ -25412,7 +25503,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L257" s="42" t="n">
+      <c r="L257" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M257" s="40" t="inlineStr">
@@ -25504,7 +25595,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L258" s="42" t="n">
+      <c r="L258" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M258" s="40" t="inlineStr">
@@ -25596,7 +25687,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L259" s="42" t="n">
+      <c r="L259" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M259" s="40" t="inlineStr">
@@ -25688,7 +25779,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L260" s="42" t="n">
+      <c r="L260" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M260" s="40" t="inlineStr">
@@ -25780,7 +25871,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L261" s="42" t="n">
+      <c r="L261" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M261" s="40" t="inlineStr">
@@ -25872,7 +25963,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L262" s="42" t="n">
+      <c r="L262" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M262" s="40" t="inlineStr">
@@ -25964,7 +26055,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L263" s="42" t="n">
+      <c r="L263" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M263" s="40" t="inlineStr">
@@ -26056,7 +26147,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L264" s="42" t="n">
+      <c r="L264" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M264" s="40" t="inlineStr">
@@ -26148,7 +26239,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L265" s="42" t="n">
+      <c r="L265" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M265" s="40" t="inlineStr">
@@ -26240,7 +26331,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L266" s="42" t="n">
+      <c r="L266" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M266" s="40" t="inlineStr">
@@ -26332,7 +26423,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L267" s="42" t="n">
+      <c r="L267" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M267" s="40" t="inlineStr">
@@ -26424,7 +26515,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L268" s="42" t="n">
+      <c r="L268" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M268" s="40" t="inlineStr">
@@ -26516,7 +26607,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L269" s="42" t="n">
+      <c r="L269" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M269" s="40" t="inlineStr">
@@ -26608,7 +26699,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L270" s="42" t="n">
+      <c r="L270" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M270" s="40" t="inlineStr">
@@ -26700,7 +26791,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L271" s="42" t="n">
+      <c r="L271" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M271" s="40" t="inlineStr">
@@ -26792,7 +26883,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L272" s="42" t="n">
+      <c r="L272" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M272" s="40" t="inlineStr">
@@ -26884,7 +26975,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L273" s="42" t="n">
+      <c r="L273" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M273" s="40" t="inlineStr">
@@ -26976,7 +27067,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L274" s="42" t="n">
+      <c r="L274" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M274" s="40" t="inlineStr">
@@ -27068,7 +27159,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L275" s="42" t="n">
+      <c r="L275" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M275" s="40" t="inlineStr">
@@ -27160,7 +27251,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L276" s="42" t="n">
+      <c r="L276" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M276" s="40" t="inlineStr">
@@ -27252,7 +27343,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L277" s="42" t="n">
+      <c r="L277" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M277" s="40" t="inlineStr">
@@ -27344,7 +27435,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L278" s="42" t="n">
+      <c r="L278" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M278" s="40" t="inlineStr">
@@ -27436,7 +27527,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L279" s="42" t="n">
+      <c r="L279" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M279" s="40" t="inlineStr">
@@ -27530,7 +27621,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="L280" s="42" t="n">
+      <c r="L280" s="60" t="n">
         <v>15</v>
       </c>
       <c r="M280" s="40" t="inlineStr">
@@ -27622,7 +27713,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L281" s="42" t="n">
+      <c r="L281" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M281" s="40" t="inlineStr">
@@ -27714,7 +27805,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L282" s="42" t="n">
+      <c r="L282" s="60" t="n">
         <v>15</v>
       </c>
       <c r="M282" s="40" t="inlineStr">
@@ -27806,7 +27897,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L283" s="42" t="n">
+      <c r="L283" s="60" t="n">
         <v>10</v>
       </c>
       <c r="M283" s="40" t="inlineStr">
@@ -27898,7 +27989,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L284" s="42" t="n">
+      <c r="L284" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M284" s="40" t="inlineStr">
@@ -27990,7 +28081,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L285" s="42" t="n">
+      <c r="L285" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M285" s="40" t="inlineStr">
@@ -28082,7 +28173,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L286" s="42" t="n">
+      <c r="L286" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M286" s="40" t="inlineStr">
@@ -28174,7 +28265,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L287" s="42" t="n">
+      <c r="L287" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M287" s="40" t="inlineStr">
@@ -28266,7 +28357,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L288" s="42" t="n">
+      <c r="L288" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M288" s="40" t="inlineStr">
@@ -28358,7 +28449,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L289" s="42" t="n">
+      <c r="L289" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M289" s="40" t="inlineStr">
@@ -28450,7 +28541,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L290" s="42" t="n">
+      <c r="L290" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M290" s="40" t="inlineStr">
@@ -28542,7 +28633,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L291" s="42" t="n">
+      <c r="L291" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M291" s="40" t="inlineStr">
@@ -28634,7 +28725,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L292" s="42" t="n">
+      <c r="L292" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M292" s="40" t="inlineStr">
@@ -28726,7 +28817,7 @@
           <t>RedBox - ريدبوكس</t>
         </is>
       </c>
-      <c r="L293" s="42" t="n">
+      <c r="L293" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M293" s="40" t="inlineStr">
@@ -28818,7 +28909,7 @@
           <t>ارامكس - ARAMEX</t>
         </is>
       </c>
-      <c r="L294" s="42" t="n">
+      <c r="L294" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M294" s="40" t="inlineStr">
@@ -28910,7 +29001,7 @@
           <t>RedBox - ريدبوكس</t>
         </is>
       </c>
-      <c r="L295" s="42" t="n">
+      <c r="L295" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M295" s="40" t="inlineStr">
@@ -29002,7 +29093,7 @@
           <t>aramex ( استلام من الفرع )</t>
         </is>
       </c>
-      <c r="L296" s="42" t="n">
+      <c r="L296" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M296" s="40" t="inlineStr">
@@ -29094,7 +29185,7 @@
           <t>RedBox - ريدبوكس</t>
         </is>
       </c>
-      <c r="L297" s="42" t="n">
+      <c r="L297" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M297" s="40" t="inlineStr">
@@ -29188,7 +29279,7 @@
           <t>JT Express</t>
         </is>
       </c>
-      <c r="L298" s="42" t="n">
+      <c r="L298" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M298" s="40" t="inlineStr">
@@ -29282,7 +29373,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="L299" s="42" t="n">
+      <c r="L299" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M299" s="40" t="inlineStr">
@@ -29374,7 +29465,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L300" s="42" t="n">
+      <c r="L300" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M300" s="40" t="inlineStr">
@@ -29466,7 +29557,7 @@
           <t>RedBox - ريدبوكس</t>
         </is>
       </c>
-      <c r="L301" s="42" t="n">
+      <c r="L301" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M301" s="40" t="inlineStr">
@@ -29558,7 +29649,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L302" s="42" t="n">
+      <c r="L302" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M302" s="40" t="inlineStr">
@@ -29650,7 +29741,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L303" s="42" t="n">
+      <c r="L303" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M303" s="40" t="inlineStr">
@@ -29742,7 +29833,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L304" s="42" t="n">
+      <c r="L304" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M304" s="40" t="inlineStr">
@@ -29834,7 +29925,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L305" s="42" t="n">
+      <c r="L305" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M305" s="40" t="inlineStr">
@@ -29926,7 +30017,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L306" s="42" t="n">
+      <c r="L306" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M306" s="40" t="inlineStr">
@@ -30018,7 +30109,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L307" s="42" t="n">
+      <c r="L307" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M307" s="40" t="inlineStr">
@@ -30112,7 +30203,7 @@
           <t>JT Express</t>
         </is>
       </c>
-      <c r="L308" s="42" t="n">
+      <c r="L308" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M308" s="40" t="inlineStr">
@@ -30204,7 +30295,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L309" s="42" t="n">
+      <c r="L309" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M309" s="40" t="inlineStr">
@@ -30298,7 +30389,7 @@
           <t>غير محدد</t>
         </is>
       </c>
-      <c r="L310" s="42" t="n">
+      <c r="L310" s="60" t="n">
         <v>15</v>
       </c>
       <c r="M310" s="40" t="inlineStr">
@@ -30390,7 +30481,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L311" s="42" t="n">
+      <c r="L311" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M311" s="40" t="inlineStr">
@@ -30484,7 +30575,7 @@
           <t>ارامكس - ARAMEX</t>
         </is>
       </c>
-      <c r="L312" s="42" t="n">
+      <c r="L312" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M312" s="40" t="inlineStr">
@@ -30578,7 +30669,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L313" s="42" t="n">
+      <c r="L313" s="60" t="n">
         <v>0.5</v>
       </c>
       <c r="M313" s="40" t="inlineStr">
@@ -30672,7 +30763,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L314" s="42" t="n">
+      <c r="L314" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M314" s="40" t="inlineStr">
@@ -30766,7 +30857,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L315" s="42" t="n">
+      <c r="L315" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M315" s="40" t="inlineStr">
@@ -30860,7 +30951,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L316" s="42" t="n">
+      <c r="L316" s="60" t="n">
         <v>10</v>
       </c>
       <c r="M316" s="40" t="inlineStr">
@@ -30954,7 +31045,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L317" s="42" t="n">
+      <c r="L317" s="60" t="n">
         <v>10</v>
       </c>
       <c r="M317" s="40" t="inlineStr">
@@ -31048,7 +31139,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L318" s="42" t="n">
+      <c r="L318" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M318" s="40" t="inlineStr">
@@ -31142,7 +31233,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L319" s="42" t="n">
+      <c r="L319" s="60" t="n">
         <v>3</v>
       </c>
       <c r="M319" s="40" t="inlineStr">
@@ -31236,7 +31327,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L320" s="42" t="n">
+      <c r="L320" s="60" t="n">
         <v>2</v>
       </c>
       <c r="M320" s="40" t="inlineStr">
@@ -31330,7 +31421,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L321" s="42" t="n">
+      <c r="L321" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M321" s="40" t="inlineStr">
@@ -31424,7 +31515,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L322" s="42" t="n">
+      <c r="L322" s="60" t="n">
         <v>5</v>
       </c>
       <c r="M322" s="40" t="inlineStr">
@@ -31518,7 +31609,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L323" s="42" t="n">
+      <c r="L323" s="60" t="n">
         <v>10</v>
       </c>
       <c r="M323" s="40" t="inlineStr">
@@ -31612,7 +31703,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L324" s="42" t="n">
+      <c r="L324" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M324" s="40" t="inlineStr">
@@ -31706,7 +31797,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L325" s="42" t="n">
+      <c r="L325" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M325" s="40" t="inlineStr">
@@ -31800,7 +31891,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L326" s="42" t="n">
+      <c r="L326" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M326" s="40" t="inlineStr">
@@ -31894,7 +31985,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L327" s="42" t="n">
+      <c r="L327" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M327" s="40" t="inlineStr">
@@ -31988,7 +32079,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L328" s="42" t="n">
+      <c r="L328" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M328" s="40" t="inlineStr">
@@ -32082,7 +32173,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L329" s="42" t="n">
+      <c r="L329" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M329" s="40" t="inlineStr">
@@ -32176,7 +32267,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L330" s="42" t="n">
+      <c r="L330" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M330" s="40" t="inlineStr">
@@ -32270,7 +32361,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L331" s="42" t="n">
+      <c r="L331" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M331" s="40" t="inlineStr">
@@ -32364,7 +32455,7 @@
           <t>SMSA - سمسا</t>
         </is>
       </c>
-      <c r="L332" s="42" t="n">
+      <c r="L332" s="60" t="n">
         <v>1</v>
       </c>
       <c r="M332" s="40" t="inlineStr">
@@ -32856,7 +32947,7 @@
           <t>#1362</t>
         </is>
       </c>
-      <c r="B12" s="59" t="n">
+      <c r="B12" s="61" t="n">
         <v>46186.66527777778</v>
       </c>
       <c r="C12" s="40" t="inlineStr">
@@ -32894,7 +32985,7 @@
           <t>#1361</t>
         </is>
       </c>
-      <c r="B13" s="59" t="n">
+      <c r="B13" s="61" t="n">
         <v>46186.66527777778</v>
       </c>
       <c r="C13" s="40" t="inlineStr">
@@ -32932,7 +33023,7 @@
           <t>#1356</t>
         </is>
       </c>
-      <c r="B14" s="59" t="n">
+      <c r="B14" s="61" t="n">
         <v>46186.47708333333</v>
       </c>
       <c r="C14" s="40" t="inlineStr">
@@ -32970,7 +33061,7 @@
           <t>#1352</t>
         </is>
       </c>
-      <c r="B15" s="59" t="n">
+      <c r="B15" s="61" t="n">
         <v>46185.65902777778</v>
       </c>
       <c r="C15" s="40" t="inlineStr">
@@ -33008,7 +33099,7 @@
           <t>#1348</t>
         </is>
       </c>
-      <c r="B16" s="59" t="n">
+      <c r="B16" s="61" t="n">
         <v>46184.89652777778</v>
       </c>
       <c r="C16" s="40" t="inlineStr">
@@ -33046,7 +33137,7 @@
           <t>#1345</t>
         </is>
       </c>
-      <c r="B17" s="59" t="n">
+      <c r="B17" s="61" t="n">
         <v>46184.88402777778</v>
       </c>
       <c r="C17" s="40" t="inlineStr">
@@ -33084,7 +33175,7 @@
           <t>#1344</t>
         </is>
       </c>
-      <c r="B18" s="59" t="n">
+      <c r="B18" s="61" t="n">
         <v>46184.82361111111</v>
       </c>
       <c r="C18" s="40" t="inlineStr">
@@ -33122,7 +33213,7 @@
           <t>#1342</t>
         </is>
       </c>
-      <c r="B19" s="59" t="n">
+      <c r="B19" s="61" t="n">
         <v>46184.82152777778</v>
       </c>
       <c r="C19" s="40" t="inlineStr">
@@ -33160,7 +33251,7 @@
           <t>#1337</t>
         </is>
       </c>
-      <c r="B20" s="59" t="n">
+      <c r="B20" s="61" t="n">
         <v>46184.79444444444</v>
       </c>
       <c r="C20" s="40" t="inlineStr">
@@ -33198,7 +33289,7 @@
           <t>#1328</t>
         </is>
       </c>
-      <c r="B21" s="59" t="n">
+      <c r="B21" s="61" t="n">
         <v>46183.91388888889</v>
       </c>
       <c r="C21" s="40" t="inlineStr">
@@ -33236,7 +33327,7 @@
           <t>#1317</t>
         </is>
       </c>
-      <c r="B22" s="59" t="n">
+      <c r="B22" s="61" t="n">
         <v>46182.94791666666</v>
       </c>
       <c r="C22" s="40" t="inlineStr">
@@ -33274,7 +33365,7 @@
           <t>#1310</t>
         </is>
       </c>
-      <c r="B23" s="59" t="n">
+      <c r="B23" s="61" t="n">
         <v>46182.45625</v>
       </c>
       <c r="C23" s="40" t="inlineStr">
@@ -33312,7 +33403,7 @@
           <t>#1309</t>
         </is>
       </c>
-      <c r="B24" s="59" t="n">
+      <c r="B24" s="61" t="n">
         <v>46182.03611111111</v>
       </c>
       <c r="C24" s="40" t="inlineStr">
@@ -33350,7 +33441,7 @@
           <t>#1308</t>
         </is>
       </c>
-      <c r="B25" s="59" t="n">
+      <c r="B25" s="61" t="n">
         <v>46182.03541666667</v>
       </c>
       <c r="C25" s="40" t="inlineStr">
@@ -33388,7 +33479,7 @@
           <t>#1292</t>
         </is>
       </c>
-      <c r="B26" s="59" t="n">
+      <c r="B26" s="61" t="n">
         <v>46180.60833333333</v>
       </c>
       <c r="C26" s="40" t="inlineStr">
@@ -33426,7 +33517,7 @@
           <t>#1285</t>
         </is>
       </c>
-      <c r="B27" s="59" t="n">
+      <c r="B27" s="61" t="n">
         <v>46179.89375</v>
       </c>
       <c r="C27" s="40" t="inlineStr">
@@ -33464,7 +33555,7 @@
           <t>#1278</t>
         </is>
       </c>
-      <c r="B28" s="59" t="n">
+      <c r="B28" s="61" t="n">
         <v>46179.60069444445</v>
       </c>
       <c r="C28" s="40" t="inlineStr">
@@ -33502,7 +33593,7 @@
           <t>#1274</t>
         </is>
       </c>
-      <c r="B29" s="59" t="n">
+      <c r="B29" s="61" t="n">
         <v>46178.68055555555</v>
       </c>
       <c r="C29" s="40" t="inlineStr">
@@ -33538,7 +33629,7 @@
           <t>#1272</t>
         </is>
       </c>
-      <c r="B30" s="59" t="n">
+      <c r="B30" s="61" t="n">
         <v>46178.12361111111</v>
       </c>
       <c r="C30" s="40" t="inlineStr">
@@ -33576,7 +33667,7 @@
           <t>#1271</t>
         </is>
       </c>
-      <c r="B31" s="59" t="n">
+      <c r="B31" s="61" t="n">
         <v>46177.80625</v>
       </c>
       <c r="C31" s="40" t="inlineStr">
@@ -33614,7 +33705,7 @@
           <t>#1263</t>
         </is>
       </c>
-      <c r="B32" s="59" t="n">
+      <c r="B32" s="61" t="n">
         <v>46177.50833333333</v>
       </c>
       <c r="C32" s="40" t="inlineStr">
@@ -33652,7 +33743,7 @@
           <t>#1262</t>
         </is>
       </c>
-      <c r="B33" s="59" t="n">
+      <c r="B33" s="61" t="n">
         <v>46177.49027777778</v>
       </c>
       <c r="C33" s="40" t="inlineStr">
@@ -33690,7 +33781,7 @@
           <t>#1261</t>
         </is>
       </c>
-      <c r="B34" s="59" t="n">
+      <c r="B34" s="61" t="n">
         <v>46177.44652777778</v>
       </c>
       <c r="C34" s="40" t="inlineStr">
@@ -33728,7 +33819,7 @@
           <t>#1256</t>
         </is>
       </c>
-      <c r="B35" s="59" t="n">
+      <c r="B35" s="61" t="n">
         <v>46176.73194444444</v>
       </c>
       <c r="C35" s="40" t="inlineStr">
@@ -33764,7 +33855,7 @@
           <t>#1255</t>
         </is>
       </c>
-      <c r="B36" s="59" t="n">
+      <c r="B36" s="61" t="n">
         <v>46176.73125</v>
       </c>
       <c r="C36" s="40" t="inlineStr">
@@ -33800,7 +33891,7 @@
           <t>#1254</t>
         </is>
       </c>
-      <c r="B37" s="59" t="n">
+      <c r="B37" s="61" t="n">
         <v>46176.73125</v>
       </c>
       <c r="C37" s="40" t="inlineStr">
@@ -33836,7 +33927,7 @@
           <t>#1246</t>
         </is>
       </c>
-      <c r="B38" s="59" t="n">
+      <c r="B38" s="61" t="n">
         <v>46176.46805555555</v>
       </c>
       <c r="C38" s="40" t="inlineStr">
@@ -33874,7 +33965,7 @@
           <t>#1245</t>
         </is>
       </c>
-      <c r="B39" s="59" t="n">
+      <c r="B39" s="61" t="n">
         <v>46176.05347222222</v>
       </c>
       <c r="C39" s="40" t="inlineStr">
@@ -33912,7 +34003,7 @@
           <t>#1244</t>
         </is>
       </c>
-      <c r="B40" s="59" t="n">
+      <c r="B40" s="61" t="n">
         <v>46175.86875</v>
       </c>
       <c r="C40" s="40" t="inlineStr">
@@ -33950,7 +34041,7 @@
           <t>#1233</t>
         </is>
       </c>
-      <c r="B41" s="59" t="n">
+      <c r="B41" s="61" t="n">
         <v>46174.52638888889</v>
       </c>
       <c r="C41" s="40" t="inlineStr">
@@ -33988,7 +34079,7 @@
           <t>#1232</t>
         </is>
       </c>
-      <c r="B42" s="59" t="n">
+      <c r="B42" s="61" t="n">
         <v>46174.50138888889</v>
       </c>
       <c r="C42" s="40" t="inlineStr">
@@ -34026,4 +34117,192 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="62" t="inlineStr">
+        <is>
+          <t>كشف الحساب الجاري</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="63" t="inlineStr">
+        <is>
+          <t>المصدر: كشف حساب جاري PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="64" t="inlineStr">
+        <is>
+          <t>ملخص الكشف</t>
+        </is>
+      </c>
+      <c r="D3" s="64" t="inlineStr">
+        <is>
+          <t>تفاصيل سريعة</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="65" t="inlineStr">
+        <is>
+          <t>إجمالي الإيداعات</t>
+        </is>
+      </c>
+      <c r="B4" s="66" t="n">
+        <v>5632</v>
+      </c>
+      <c r="D4" s="65" t="inlineStr">
+        <is>
+          <t>عدد الإيداعات</t>
+        </is>
+      </c>
+      <c r="E4" s="66" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="65" t="inlineStr">
+        <is>
+          <t>إجمالي المصاريف</t>
+        </is>
+      </c>
+      <c r="B5" s="66" t="n">
+        <v>4463.26</v>
+      </c>
+      <c r="D5" s="65" t="inlineStr">
+        <is>
+          <t>عدد المصاريف</t>
+        </is>
+      </c>
+      <c r="E5" s="66" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="65" t="inlineStr">
+        <is>
+          <t>صافي الحركة</t>
+        </is>
+      </c>
+      <c r="B6" s="66" t="n">
+        <v>1168.74</v>
+      </c>
+      <c r="D6" s="65" t="inlineStr">
+        <is>
+          <t>الفترة</t>
+        </is>
+      </c>
+      <c r="E6" s="67" t="inlineStr">
+        <is>
+          <t>2026/06/01 - 2026/06/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="65" t="inlineStr">
+        <is>
+          <t>إجمالي رسوم الحوالات</t>
+        </is>
+      </c>
+      <c r="B7" s="68" t="n">
+        <v>1.73</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1"/>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="69" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="B9" s="69" t="inlineStr">
+        <is>
+          <t>نوع المصروف</t>
+        </is>
+      </c>
+      <c r="C9" s="69" t="inlineStr">
+        <is>
+          <t>المبلغ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="70" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B10" s="71" t="inlineStr">
+        <is>
+          <t>فاتورة 12</t>
+        </is>
+      </c>
+      <c r="C10" s="72" t="n">
+        <v>3477.39</v>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="70" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B11" s="71" t="inlineStr">
+        <is>
+          <t>رسوم فاتورة 12</t>
+        </is>
+      </c>
+      <c r="C11" s="72" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="70" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B12" s="71" t="inlineStr">
+        <is>
+          <t>فاتورة 13</t>
+        </is>
+      </c>
+      <c r="C12" s="72" t="n">
+        <v>984.14</v>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="70" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B13" s="71" t="inlineStr">
+        <is>
+          <t>رسوم فاتورة 13</t>
+        </is>
+      </c>
+      <c r="C13" s="72" t="n">
+        <v>0.58</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A9:C13"/>
+  <mergeCells count="4">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add June 16 dashboard data
</commit_message>
<xml_diff>
--- a/output/lead6_report.xlsx
+++ b/output/lead6_report.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كشف الحساب" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'تفاصيل شهر 6'!$A$1:$X$441</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'تفاصيل شهر 6'!$A$1:$X$460</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'كشف الحساب'!$A$9:$C$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -652,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -668,7 +668,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>2026-06-01 - 2026-06-15</t>
+          <t>2026-06-01 - 2026-06-16</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>440</v>
+        <v>459</v>
       </c>
       <c r="C4" s="4" t="n"/>
       <c r="D4" s="4" t="n"/>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>428</v>
+        <v>442</v>
       </c>
       <c r="C5" s="4" t="n"/>
       <c r="D5" s="4" t="n"/>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="4" t="n"/>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>1143.63</v>
+        <v>1210.18</v>
       </c>
       <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="n"/>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>6609</v>
+        <v>6859</v>
       </c>
       <c r="C10" s="4" t="n"/>
       <c r="D10" s="4" t="n"/>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>8741.889999999999</v>
+        <v>8671.389999999999</v>
       </c>
       <c r="C12" s="4" t="n"/>
       <c r="D12" s="4" t="n"/>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>8533</v>
+        <v>8783</v>
       </c>
       <c r="C13" s="4" t="n"/>
       <c r="D13" s="4" t="n"/>
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>1155.88</v>
+        <v>1222.43</v>
       </c>
       <c r="C14" s="4" t="n"/>
       <c r="D14" s="4" t="n"/>
@@ -983,10 +983,10 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C21" s="9" t="n">
-        <v>586.7999999999993</v>
+        <v>632.4399999999991</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>0</v>
@@ -995,7 +995,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>586.7999999999993</v>
+        <v>632.4399999999991</v>
       </c>
       <c r="G21" s="4" t="n"/>
       <c r="H21" s="4" t="n"/>
@@ -1031,10 +1031,10 @@
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>131.1000000000001</v>
+        <v>148.35</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>0</v>
@@ -1043,7 +1043,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>131.1000000000001</v>
+        <v>148.35</v>
       </c>
       <c r="G23" s="4" t="n"/>
       <c r="H23" s="4" t="n"/>
@@ -1055,10 +1055,10 @@
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>92.71999999999984</v>
+        <v>94.23999999999984</v>
       </c>
       <c r="D24" s="9" t="n">
         <v>0</v>
@@ -1067,7 +1067,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>92.71999999999984</v>
+        <v>94.23999999999984</v>
       </c>
       <c r="G24" s="4" t="n"/>
       <c r="H24" s="4" t="n"/>
@@ -1123,14 +1123,14 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>خلود المالكي</t>
+          <t>فهد احمد</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C27" s="9" t="n">
-        <v>5.129999999999999</v>
+        <v>7.18</v>
       </c>
       <c r="D27" s="9" t="n">
         <v>0</v>
@@ -1139,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>5.129999999999999</v>
+        <v>7.18</v>
       </c>
       <c r="G27" s="4" t="n"/>
       <c r="H27" s="4" t="n"/>
@@ -1147,14 +1147,14 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>فهد احمد</t>
+          <t>خلود المالكي</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C28" s="9" t="n">
-        <v>5.039999999999999</v>
+        <v>5.129999999999999</v>
       </c>
       <c r="D28" s="9" t="n">
         <v>0</v>
@@ -1163,7 +1163,7 @@
         <v>0</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>5.039999999999999</v>
+        <v>5.129999999999999</v>
       </c>
       <c r="G28" s="4" t="n"/>
       <c r="H28" s="4" t="n"/>
@@ -1315,10 +1315,10 @@
         </is>
       </c>
       <c r="B36" s="4" t="n">
-        <v>408</v>
+        <v>421</v>
       </c>
       <c r="C36" s="9" t="n">
-        <v>1108.299999999996</v>
+        <v>1172.709999999996</v>
       </c>
       <c r="D36" s="9" t="n">
         <v>0</v>
@@ -1327,7 +1327,7 @@
         <v>4</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>1112.299999999996</v>
+        <v>1176.709999999996</v>
       </c>
       <c r="G36" s="4" t="n"/>
       <c r="H36" s="4" t="n"/>
@@ -1383,14 +1383,14 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>SMSA ( استلام من الفرع )</t>
+          <t>aramex ( استلام من الفرع )</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C39" s="9" t="n">
-        <v>2.010000000000002</v>
+        <v>2.140000000000001</v>
       </c>
       <c r="D39" s="9" t="n">
         <v>0</v>
@@ -1399,18 +1399,32 @@
         <v>0</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>2.010000000000002</v>
+        <v>2.140000000000001</v>
       </c>
       <c r="G39" s="4" t="n"/>
       <c r="H39" s="4" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="n"/>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="4" t="n"/>
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>SMSA ( استلام من الفرع )</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="9" t="n">
+        <v>2.010000000000002</v>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="9" t="n">
+        <v>2.010000000000002</v>
+      </c>
       <c r="G40" s="4" t="n"/>
       <c r="H40" s="4" t="n"/>
     </row>
@@ -1425,11 +1439,7 @@
       <c r="H41" s="4" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>عدد الشحنات حسب الحالة</t>
-        </is>
-      </c>
+      <c r="A42" s="4" t="n"/>
       <c r="B42" s="4" t="n"/>
       <c r="C42" s="4" t="n"/>
       <c r="D42" s="4" t="n"/>
@@ -1439,16 +1449,12 @@
       <c r="H42" s="4" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>الحالة</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>العدد</t>
-        </is>
-      </c>
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>عدد الشحنات حسب الحالة</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="n"/>
       <c r="C43" s="4" t="n"/>
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="4" t="n"/>
@@ -1457,13 +1463,15 @@
       <c r="H43" s="4" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>تم التوصيل</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="n">
-        <v>221</v>
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>الحالة</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
       </c>
       <c r="C44" s="4" t="n"/>
       <c r="D44" s="4" t="n"/>
@@ -1475,11 +1483,11 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>تم الاستلام</t>
+          <t>تم التوصيل</t>
         </is>
       </c>
       <c r="B45" s="4" t="n">
-        <v>140</v>
+        <v>221</v>
       </c>
       <c r="C45" s="4" t="n"/>
       <c r="D45" s="4" t="n"/>
@@ -1491,11 +1499,11 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>مؤكد</t>
+          <t>تم الاستلام</t>
         </is>
       </c>
       <c r="B46" s="4" t="n">
-        <v>47</v>
+        <v>151</v>
       </c>
       <c r="C46" s="4" t="n"/>
       <c r="D46" s="4" t="n"/>
@@ -1507,11 +1515,11 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>قيد الشحن</t>
+          <t>مؤكد</t>
         </is>
       </c>
       <c r="B47" s="4" t="n">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C47" s="4" t="n"/>
       <c r="D47" s="4" t="n"/>
@@ -1523,11 +1531,11 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>مسودة</t>
+          <t>قيد الشحن</t>
         </is>
       </c>
       <c r="B48" s="4" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C48" s="4" t="n"/>
       <c r="D48" s="4" t="n"/>
@@ -1539,11 +1547,11 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>ملغي</t>
+          <t>مسودة</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C49" s="4" t="n"/>
       <c r="D49" s="4" t="n"/>
@@ -1551,6 +1559,22 @@
       <c r="F49" s="4" t="n"/>
       <c r="G49" s="4" t="n"/>
       <c r="H49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>ملغي</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C50" s="4" t="n"/>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1566,7 +1590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:X443"/>
+  <dimension ref="A1:X462"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -42259,32 +42283,1786 @@
         <v>441</v>
       </c>
     </row>
+    <row r="442">
+      <c r="A442" s="10" t="n">
+        <v>2052</v>
+      </c>
+      <c r="B442" s="10" t="inlineStr">
+        <is>
+          <t>غير محدد</t>
+        </is>
+      </c>
+      <c r="C442" s="10" t="inlineStr">
+        <is>
+          <t>ابو خالد</t>
+        </is>
+      </c>
+      <c r="D442" s="10" t="inlineStr">
+        <is>
+          <t>ابو خالد</t>
+        </is>
+      </c>
+      <c r="E442" s="10" t="inlineStr">
+        <is>
+          <t>Jamil Ali</t>
+        </is>
+      </c>
+      <c r="F442" s="10" t="inlineStr">
+        <is>
+          <t>مكة المكرمة</t>
+        </is>
+      </c>
+      <c r="G442" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H442" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I442" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="J442" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K442" s="10" t="inlineStr">
+        <is>
+          <t>غير محدد</t>
+        </is>
+      </c>
+      <c r="L442" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M442" s="10" t="inlineStr">
+        <is>
+          <t>مسودة</t>
+        </is>
+      </c>
+      <c r="N442" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O442" s="10" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P442" s="10" t="inlineStr">
+        <is>
+          <t>غير موجود في شيت الأسعار / غير موجود في شيت الأسعار</t>
+        </is>
+      </c>
+      <c r="Q442" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R442" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S442" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T442" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U442" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V442" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W442" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X442" s="10" t="n">
+        <v>460</v>
+      </c>
+    </row>
     <row r="443">
-      <c r="P443" s="6" t="inlineStr">
+      <c r="A443" s="10" t="n">
+        <v>2053</v>
+      </c>
+      <c r="B443" s="10" t="n">
+        <v>291655363647</v>
+      </c>
+      <c r="C443" s="10" t="inlineStr">
+        <is>
+          <t>مؤسسة اواني القيصرية التجارية</t>
+        </is>
+      </c>
+      <c r="D443" s="10" t="inlineStr">
+        <is>
+          <t>متجر اواني</t>
+        </is>
+      </c>
+      <c r="E443" s="10" t="inlineStr">
+        <is>
+          <t>سارا</t>
+        </is>
+      </c>
+      <c r="F443" s="10" t="inlineStr">
+        <is>
+          <t>الباحة</t>
+        </is>
+      </c>
+      <c r="G443" s="11" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="H443" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I443" s="11" t="n">
+        <v>211</v>
+      </c>
+      <c r="J443" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K443" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L443" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="M443" s="10" t="inlineStr">
+        <is>
+          <t>تم الاستلام</t>
+        </is>
+      </c>
+      <c r="N443" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O443" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P443" s="10" t="inlineStr">
+        <is>
+          <t>مؤسسة اواني القيصرية التجارية / مؤسسة اواني القيصرية التجارية</t>
+        </is>
+      </c>
+      <c r="Q443" s="11" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="R443" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S443" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T443" s="11" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="U443" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V443" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W443" s="11" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="X443" s="10" t="n">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="10" t="n">
+        <v>2054</v>
+      </c>
+      <c r="B444" s="10" t="n">
+        <v>291655440347</v>
+      </c>
+      <c r="C444" s="10" t="inlineStr">
+        <is>
+          <t>احمد محمد بن عبدالله الرزق</t>
+        </is>
+      </c>
+      <c r="D444" s="10" t="inlineStr">
+        <is>
+          <t>متجر مقام الصبا | للالات الموسيقية</t>
+        </is>
+      </c>
+      <c r="E444" s="10" t="inlineStr">
+        <is>
+          <t>تركي الدوسري</t>
+        </is>
+      </c>
+      <c r="F444" s="10" t="inlineStr">
+        <is>
+          <t>Al Sulaiyl (Wadi al-Dawasir)</t>
+        </is>
+      </c>
+      <c r="G444" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H444" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I444" s="11" t="n">
+        <v>299</v>
+      </c>
+      <c r="J444" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K444" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L444" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M444" s="10" t="inlineStr">
+        <is>
+          <t>تم الاستلام</t>
+        </is>
+      </c>
+      <c r="N444" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O444" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P444" s="10" t="inlineStr">
+        <is>
+          <t>سمسا / سمسا</t>
+        </is>
+      </c>
+      <c r="Q444" s="11" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="R444" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S444" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T444" s="11" t="n">
+        <v>3.449999999999999</v>
+      </c>
+      <c r="U444" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V444" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W444" s="11" t="n">
+        <v>3.449999999999999</v>
+      </c>
+      <c r="X444" s="10" t="n">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="10" t="n">
+        <v>2055</v>
+      </c>
+      <c r="B445" s="10" t="n">
+        <v>291655440325</v>
+      </c>
+      <c r="C445" s="10" t="inlineStr">
+        <is>
+          <t>احمد محمد بن عبدالله الرزق</t>
+        </is>
+      </c>
+      <c r="D445" s="10" t="inlineStr">
+        <is>
+          <t>متجر مقام الصبا | للالات الموسيقية</t>
+        </is>
+      </c>
+      <c r="E445" s="10" t="inlineStr">
+        <is>
+          <t>Tbrjl 1</t>
+        </is>
+      </c>
+      <c r="F445" s="10" t="inlineStr">
+        <is>
+          <t>Ar Rass</t>
+        </is>
+      </c>
+      <c r="G445" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H445" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I445" s="11" t="n">
+        <v>330</v>
+      </c>
+      <c r="J445" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K445" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L445" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M445" s="10" t="inlineStr">
+        <is>
+          <t>تم الاستلام</t>
+        </is>
+      </c>
+      <c r="N445" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O445" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P445" s="10" t="inlineStr">
+        <is>
+          <t>سمسا / سمسا</t>
+        </is>
+      </c>
+      <c r="Q445" s="11" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="R445" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S445" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T445" s="11" t="n">
+        <v>3.449999999999999</v>
+      </c>
+      <c r="U445" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V445" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W445" s="11" t="n">
+        <v>3.449999999999999</v>
+      </c>
+      <c r="X445" s="10" t="n">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="10" t="n">
+        <v>2056</v>
+      </c>
+      <c r="B446" s="10" t="n">
+        <v>291655440336</v>
+      </c>
+      <c r="C446" s="10" t="inlineStr">
+        <is>
+          <t>احمد محمد بن عبدالله الرزق</t>
+        </is>
+      </c>
+      <c r="D446" s="10" t="inlineStr">
+        <is>
+          <t>متجر مقام الصبا | للالات الموسيقية</t>
+        </is>
+      </c>
+      <c r="E446" s="10" t="inlineStr">
+        <is>
+          <t>يحيئ احمد الزهراني</t>
+        </is>
+      </c>
+      <c r="F446" s="10" t="inlineStr">
+        <is>
+          <t>Dhahran</t>
+        </is>
+      </c>
+      <c r="G446" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H446" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I446" s="11" t="n">
+        <v>79</v>
+      </c>
+      <c r="J446" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K446" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L446" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M446" s="10" t="inlineStr">
+        <is>
+          <t>قيد الشحن</t>
+        </is>
+      </c>
+      <c r="N446" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O446" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P446" s="10" t="inlineStr">
+        <is>
+          <t>سمسا / سمسا</t>
+        </is>
+      </c>
+      <c r="Q446" s="11" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="R446" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S446" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T446" s="11" t="n">
+        <v>3.449999999999999</v>
+      </c>
+      <c r="U446" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V446" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W446" s="11" t="n">
+        <v>3.449999999999999</v>
+      </c>
+      <c r="X446" s="10" t="n">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="10" t="n">
+        <v>2057</v>
+      </c>
+      <c r="B447" s="10" t="n">
+        <v>291655440358</v>
+      </c>
+      <c r="C447" s="10" t="inlineStr">
+        <is>
+          <t>احمد محمد بن عبدالله الرزق</t>
+        </is>
+      </c>
+      <c r="D447" s="10" t="inlineStr">
+        <is>
+          <t>متجر مقام الصبا | للالات الموسيقية</t>
+        </is>
+      </c>
+      <c r="E447" s="10" t="inlineStr">
+        <is>
+          <t>سليم محمد سليم محمد العطوي</t>
+        </is>
+      </c>
+      <c r="F447" s="10" t="inlineStr">
+        <is>
+          <t>Tabuk</t>
+        </is>
+      </c>
+      <c r="G447" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H447" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I447" s="11" t="n">
+        <v>258</v>
+      </c>
+      <c r="J447" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K447" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L447" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M447" s="10" t="inlineStr">
+        <is>
+          <t>تم الاستلام</t>
+        </is>
+      </c>
+      <c r="N447" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O447" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P447" s="10" t="inlineStr">
+        <is>
+          <t>سمسا / سمسا</t>
+        </is>
+      </c>
+      <c r="Q447" s="11" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="R447" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S447" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T447" s="11" t="n">
+        <v>3.449999999999999</v>
+      </c>
+      <c r="U447" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V447" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W447" s="11" t="n">
+        <v>3.449999999999999</v>
+      </c>
+      <c r="X447" s="10" t="n">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="10" t="n">
+        <v>2058</v>
+      </c>
+      <c r="B448" s="10" t="n">
+        <v>291655440369</v>
+      </c>
+      <c r="C448" s="10" t="inlineStr">
+        <is>
+          <t>احمد محمد بن عبدالله الرزق</t>
+        </is>
+      </c>
+      <c r="D448" s="10" t="inlineStr">
+        <is>
+          <t>متجر مقام الصبا | للالات الموسيقية</t>
+        </is>
+      </c>
+      <c r="E448" s="10" t="inlineStr">
+        <is>
+          <t>Bee</t>
+        </is>
+      </c>
+      <c r="F448" s="10" t="inlineStr">
+        <is>
+          <t>Taif</t>
+        </is>
+      </c>
+      <c r="G448" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H448" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I448" s="11" t="n">
+        <v>499</v>
+      </c>
+      <c r="J448" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K448" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L448" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M448" s="10" t="inlineStr">
+        <is>
+          <t>مؤكد</t>
+        </is>
+      </c>
+      <c r="N448" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O448" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P448" s="10" t="inlineStr">
+        <is>
+          <t>سمسا / سمسا</t>
+        </is>
+      </c>
+      <c r="Q448" s="11" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="R448" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S448" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T448" s="11" t="n">
+        <v>3.449999999999999</v>
+      </c>
+      <c r="U448" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V448" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W448" s="11" t="n">
+        <v>3.449999999999999</v>
+      </c>
+      <c r="X448" s="10" t="n">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="10" t="n">
+        <v>2059</v>
+      </c>
+      <c r="B449" s="10" t="n">
+        <v>50837298492</v>
+      </c>
+      <c r="C449" s="10" t="inlineStr">
+        <is>
+          <t>فهد احمد</t>
+        </is>
+      </c>
+      <c r="D449" s="10" t="inlineStr">
+        <is>
+          <t>الرئيسي</t>
+        </is>
+      </c>
+      <c r="E449" s="10" t="inlineStr">
+        <is>
+          <t>علي انور زبيدي</t>
+        </is>
+      </c>
+      <c r="F449" s="10" t="inlineStr">
+        <is>
+          <t>أبو عريش</t>
+        </is>
+      </c>
+      <c r="G449" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="H449" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I449" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="J449" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K449" s="10" t="inlineStr">
+        <is>
+          <t>aramex ( استلام من الفرع )</t>
+        </is>
+      </c>
+      <c r="L449" s="26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M449" s="10" t="inlineStr">
+        <is>
+          <t>مؤكد</t>
+        </is>
+      </c>
+      <c r="N449" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O449" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P449" s="10" t="inlineStr">
+        <is>
+          <t>ارامكس استلام / ارامكس استلام</t>
+        </is>
+      </c>
+      <c r="Q449" s="11" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="R449" s="11" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="S449" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T449" s="11" t="n">
+        <v>2.140000000000001</v>
+      </c>
+      <c r="U449" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V449" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W449" s="11" t="n">
+        <v>2.140000000000001</v>
+      </c>
+      <c r="X449" s="10" t="n">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="10" t="n">
+        <v>2060</v>
+      </c>
+      <c r="B450" s="10" t="inlineStr">
+        <is>
+          <t>غير محدد</t>
+        </is>
+      </c>
+      <c r="C450" s="10" t="inlineStr">
+        <is>
+          <t>نوف مرزوق العتيبي</t>
+        </is>
+      </c>
+      <c r="D450" s="10" t="inlineStr">
+        <is>
+          <t>نوف مرزوق العتيبي</t>
+        </is>
+      </c>
+      <c r="E450" s="10" t="inlineStr">
+        <is>
+          <t>مزنه العتيبي</t>
+        </is>
+      </c>
+      <c r="F450" s="10" t="inlineStr">
+        <is>
+          <t>القويعية</t>
+        </is>
+      </c>
+      <c r="G450" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H450" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I450" s="11" t="n">
+        <v>205</v>
+      </c>
+      <c r="J450" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K450" s="10" t="inlineStr">
+        <is>
+          <t>غير محدد</t>
+        </is>
+      </c>
+      <c r="L450" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M450" s="10" t="inlineStr">
+        <is>
+          <t>مسودة</t>
+        </is>
+      </c>
+      <c r="N450" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O450" s="10" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P450" s="10" t="inlineStr">
+        <is>
+          <t>غير موجود في شيت الأسعار / غير موجود في شيت الأسعار</t>
+        </is>
+      </c>
+      <c r="Q450" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R450" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S450" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T450" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U450" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V450" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W450" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X450" s="10" t="n">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="10" t="n">
+        <v>2061</v>
+      </c>
+      <c r="B451" s="10" t="n">
+        <v>50837307511</v>
+      </c>
+      <c r="C451" s="10" t="inlineStr">
+        <is>
+          <t>ليد إكسبرس</t>
+        </is>
+      </c>
+      <c r="D451" s="10" t="inlineStr">
+        <is>
+          <t>Lead Express</t>
+        </is>
+      </c>
+      <c r="E451" s="10" t="inlineStr">
+        <is>
+          <t>LEAD EXPRESS</t>
+        </is>
+      </c>
+      <c r="F451" s="10" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="G451" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="H451" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I451" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J451" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K451" s="10" t="inlineStr">
+        <is>
+          <t>aramex ( استلام من الفرع )</t>
+        </is>
+      </c>
+      <c r="L451" s="26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M451" s="10" t="inlineStr">
+        <is>
+          <t>ملغي</t>
+        </is>
+      </c>
+      <c r="N451" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O451" s="10" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P451" s="10" t="inlineStr">
+        <is>
+          <t>ارامكس استلام / ارامكس استلام</t>
+        </is>
+      </c>
+      <c r="Q451" s="11" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="R451" s="11" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="S451" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T451" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U451" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V451" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W451" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X451" s="10" t="n">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="10" t="n">
+        <v>2062</v>
+      </c>
+      <c r="B452" s="10" t="n">
+        <v>291655470433</v>
+      </c>
+      <c r="C452" s="10" t="inlineStr">
+        <is>
+          <t>ليد إكسبرس</t>
+        </is>
+      </c>
+      <c r="D452" s="10" t="inlineStr">
+        <is>
+          <t>Lead Express</t>
+        </is>
+      </c>
+      <c r="E452" s="10" t="inlineStr">
+        <is>
+          <t>LEAD EXPRESS</t>
+        </is>
+      </c>
+      <c r="F452" s="10" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="G452" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H452" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I452" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J452" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K452" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L452" s="26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M452" s="10" t="inlineStr">
+        <is>
+          <t>ملغي</t>
+        </is>
+      </c>
+      <c r="N452" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O452" s="10" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P452" s="10" t="inlineStr">
+        <is>
+          <t>سمسا / سمسا</t>
+        </is>
+      </c>
+      <c r="Q452" s="11" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="R452" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S452" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T452" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U452" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V452" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W452" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X452" s="10" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="10" t="n">
+        <v>2064</v>
+      </c>
+      <c r="B453" s="10" t="n">
+        <v>291655494955</v>
+      </c>
+      <c r="C453" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="D453" s="10" t="inlineStr">
+        <is>
+          <t>الوتر السابع للألأت الموسيقية</t>
+        </is>
+      </c>
+      <c r="E453" s="10" t="inlineStr">
+        <is>
+          <t>وعد</t>
+        </is>
+      </c>
+      <c r="F453" s="10" t="inlineStr">
+        <is>
+          <t>Dammam</t>
+        </is>
+      </c>
+      <c r="G453" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H453" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I453" s="11" t="n">
+        <v>395</v>
+      </c>
+      <c r="J453" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K453" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L453" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M453" s="10" t="inlineStr">
+        <is>
+          <t>تم الاستلام</t>
+        </is>
+      </c>
+      <c r="N453" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O453" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P453" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري / عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="Q453" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="R453" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S453" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T453" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="U453" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V453" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W453" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="X453" s="10" t="n">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="10" t="n">
+        <v>2065</v>
+      </c>
+      <c r="B454" s="10" t="n">
+        <v>291655494933</v>
+      </c>
+      <c r="C454" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="D454" s="10" t="inlineStr">
+        <is>
+          <t>الوتر السابع للألأت الموسيقية</t>
+        </is>
+      </c>
+      <c r="E454" s="10" t="inlineStr">
+        <is>
+          <t>علي حماده</t>
+        </is>
+      </c>
+      <c r="F454" s="10" t="inlineStr">
+        <is>
+          <t>Al Jubail</t>
+        </is>
+      </c>
+      <c r="G454" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H454" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I454" s="11" t="n">
+        <v>650</v>
+      </c>
+      <c r="J454" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K454" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L454" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M454" s="10" t="inlineStr">
+        <is>
+          <t>تم الاستلام</t>
+        </is>
+      </c>
+      <c r="N454" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O454" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P454" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري / عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="Q454" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="R454" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S454" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T454" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="U454" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V454" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W454" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="X454" s="10" t="n">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="10" t="n">
+        <v>2066</v>
+      </c>
+      <c r="B455" s="10" t="n">
+        <v>291655494977</v>
+      </c>
+      <c r="C455" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="D455" s="10" t="inlineStr">
+        <is>
+          <t>الوتر السابع للألأت الموسيقية</t>
+        </is>
+      </c>
+      <c r="E455" s="10" t="inlineStr">
+        <is>
+          <t>محمد ساري الجهني</t>
+        </is>
+      </c>
+      <c r="F455" s="10" t="inlineStr">
+        <is>
+          <t>Umluj</t>
+        </is>
+      </c>
+      <c r="G455" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H455" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I455" s="11" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J455" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K455" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L455" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M455" s="10" t="inlineStr">
+        <is>
+          <t>تم الاستلام</t>
+        </is>
+      </c>
+      <c r="N455" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O455" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P455" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري / عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="Q455" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="R455" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S455" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T455" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="U455" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V455" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W455" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="X455" s="10" t="n">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="10" t="n">
+        <v>2067</v>
+      </c>
+      <c r="B456" s="10" t="n">
+        <v>291655494999</v>
+      </c>
+      <c r="C456" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="D456" s="10" t="inlineStr">
+        <is>
+          <t>الوتر السابع للألأت الموسيقية</t>
+        </is>
+      </c>
+      <c r="E456" s="10" t="inlineStr">
+        <is>
+          <t>عبدالله الاسلمي</t>
+        </is>
+      </c>
+      <c r="F456" s="10" t="inlineStr">
+        <is>
+          <t>Hafar Al Batin</t>
+        </is>
+      </c>
+      <c r="G456" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H456" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I456" s="11" t="n">
+        <v>395</v>
+      </c>
+      <c r="J456" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K456" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L456" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M456" s="10" t="inlineStr">
+        <is>
+          <t>تم الاستلام</t>
+        </is>
+      </c>
+      <c r="N456" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O456" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P456" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري / عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="Q456" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="R456" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S456" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T456" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="U456" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V456" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W456" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="X456" s="10" t="n">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="10" t="n">
+        <v>2068</v>
+      </c>
+      <c r="B457" s="10" t="n">
+        <v>291655494944</v>
+      </c>
+      <c r="C457" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="D457" s="10" t="inlineStr">
+        <is>
+          <t>الوتر السابع للألأت الموسيقية</t>
+        </is>
+      </c>
+      <c r="E457" s="10" t="inlineStr">
+        <is>
+          <t>مراد سعيد</t>
+        </is>
+      </c>
+      <c r="F457" s="10" t="inlineStr">
+        <is>
+          <t>Jeddah</t>
+        </is>
+      </c>
+      <c r="G457" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H457" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I457" s="11" t="n">
+        <v>480</v>
+      </c>
+      <c r="J457" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K457" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L457" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M457" s="10" t="inlineStr">
+        <is>
+          <t>تم الاستلام</t>
+        </is>
+      </c>
+      <c r="N457" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O457" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P457" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري / عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="Q457" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="R457" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S457" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T457" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="U457" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V457" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W457" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="X457" s="10" t="n">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="10" t="n">
+        <v>2069</v>
+      </c>
+      <c r="B458" s="10" t="n">
+        <v>291655501300</v>
+      </c>
+      <c r="C458" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="D458" s="10" t="inlineStr">
+        <is>
+          <t>الوتر السابع للألأت الموسيقية</t>
+        </is>
+      </c>
+      <c r="E458" s="10" t="inlineStr">
+        <is>
+          <t>امجد سلمان السياط</t>
+        </is>
+      </c>
+      <c r="F458" s="10" t="inlineStr">
+        <is>
+          <t>سكاكا</t>
+        </is>
+      </c>
+      <c r="G458" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H458" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I458" s="11" t="n">
+        <v>360</v>
+      </c>
+      <c r="J458" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K458" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L458" s="26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M458" s="10" t="inlineStr">
+        <is>
+          <t>تم الاستلام</t>
+        </is>
+      </c>
+      <c r="N458" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O458" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P458" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري / عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="Q458" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="R458" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S458" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T458" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="U458" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V458" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W458" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="X458" s="10" t="n">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="10" t="n">
+        <v>2070</v>
+      </c>
+      <c r="B459" s="10" t="n">
+        <v>291655494966</v>
+      </c>
+      <c r="C459" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="D459" s="10" t="inlineStr">
+        <is>
+          <t>الوتر السابع للألأت الموسيقية</t>
+        </is>
+      </c>
+      <c r="E459" s="10" t="inlineStr">
+        <is>
+          <t>مهند العنزي</t>
+        </is>
+      </c>
+      <c r="F459" s="10" t="inlineStr">
+        <is>
+          <t>TAYMA&amp;#039;</t>
+        </is>
+      </c>
+      <c r="G459" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H459" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I459" s="11" t="n">
+        <v>485</v>
+      </c>
+      <c r="J459" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K459" s="10" t="inlineStr">
+        <is>
+          <t>SMSA - سمسا</t>
+        </is>
+      </c>
+      <c r="L459" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M459" s="10" t="inlineStr">
+        <is>
+          <t>تم الاستلام</t>
+        </is>
+      </c>
+      <c r="N459" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O459" s="10" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="P459" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري / عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="Q459" s="11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="R459" s="11" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="S459" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T459" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="U459" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V459" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W459" s="11" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="X459" s="10" t="n">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="10" t="n">
+        <v>2071</v>
+      </c>
+      <c r="B460" s="10" t="inlineStr">
+        <is>
+          <t>ara20260616214211002071</t>
+        </is>
+      </c>
+      <c r="C460" s="10" t="inlineStr">
+        <is>
+          <t>ليد إكسبرس</t>
+        </is>
+      </c>
+      <c r="D460" s="10" t="inlineStr">
+        <is>
+          <t>Lead Express</t>
+        </is>
+      </c>
+      <c r="E460" s="10" t="inlineStr">
+        <is>
+          <t>LEAD EXPRESS</t>
+        </is>
+      </c>
+      <c r="F460" s="10" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="G460" s="11" t="n">
+        <v>23</v>
+      </c>
+      <c r="H460" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I460" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J460" s="10" t="inlineStr">
+        <is>
+          <t>💰 مسبق</t>
+        </is>
+      </c>
+      <c r="K460" s="10" t="inlineStr">
+        <is>
+          <t>أرامكس (Treek)</t>
+        </is>
+      </c>
+      <c r="L460" s="26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M460" s="10" t="inlineStr">
+        <is>
+          <t>ملغي</t>
+        </is>
+      </c>
+      <c r="N460" s="13" t="n">
+        <v>46189</v>
+      </c>
+      <c r="O460" s="10" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P460" s="10" t="inlineStr">
+        <is>
+          <t>شيت الشحنات / غير موجود في شيت الأسعار</t>
+        </is>
+      </c>
+      <c r="Q460" s="11" t="n">
+        <v>19.55</v>
+      </c>
+      <c r="R460" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S460" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T460" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U460" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V460" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W460" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X460" s="10" t="n">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="P462" s="6" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="Q443" s="7" t="n">
-        <v>8493.220000000001</v>
-      </c>
-      <c r="R443" s="7" t="n">
-        <v>7322.75</v>
-      </c>
-      <c r="S443" s="15" t="n"/>
-      <c r="T443" s="7" t="n">
-        <v>1143.63</v>
-      </c>
-      <c r="U443" s="7" t="n">
+      <c r="Q462" s="7" t="n">
+        <v>8853.130000000001</v>
+      </c>
+      <c r="R462" s="7" t="n">
+        <v>7590.97</v>
+      </c>
+      <c r="S462" s="15" t="n"/>
+      <c r="T462" s="7" t="n">
+        <v>1210.18</v>
+      </c>
+      <c r="U462" s="7" t="n">
         <v>4.25</v>
       </c>
-      <c r="V443" s="15" t="n"/>
-      <c r="W443" s="7" t="n">
-        <v>1155.88</v>
+      <c r="V462" s="15" t="n"/>
+      <c r="W462" s="7" t="n">
+        <v>1222.43</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X441"/>
+  <autoFilter ref="A1:X460"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -42523,7 +44301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -42573,10 +44351,10 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>6609</v>
+        <v>6859</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -42625,10 +44403,10 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>103</v>
+        <v>169.5</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
@@ -42638,10 +44416,10 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>8533</v>
+        <v>8783</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1"/>
@@ -43860,62 +45638,62 @@
     <row r="43" ht="24" customHeight="1">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>#1382</t>
+          <t>#1409</t>
         </is>
       </c>
       <c r="B43" s="27" t="n">
-        <v>41816.91944444444</v>
+        <v>42547.90486111111</v>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>فارس احمد</t>
+          <t>ليد إكسبرس</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>إيداع</t>
+          <t>استرداد</t>
         </is>
       </c>
       <c r="E43" s="11" t="n">
-        <v>252</v>
+        <v>23</v>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t>شحن رصيد عبر تحويل بنكي - مرجع: 132_1781463851_d66934a2.jpeg [صورة: 132_1781463851_d66934a2.jpeg]</t>
+          <t>استرداد تكلفة شحن - إلغاء طلب #2071</t>
         </is>
       </c>
       <c r="G43" s="10" t="n"/>
       <c r="H43" s="10" t="inlineStr">
         <is>
-          <t>البنك</t>
+          <t>أخرى</t>
         </is>
       </c>
     </row>
     <row r="44" ht="24" customHeight="1">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>#1380</t>
+          <t>#1408</t>
         </is>
       </c>
       <c r="B44" s="27" t="n">
-        <v>41816.74444444444</v>
+        <v>42547.90416666667</v>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>مؤسسة اواني القيصرية التجارية</t>
+          <t>ليد إكسبرس</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>admin_deduction</t>
+          <t>شحن</t>
         </is>
       </c>
       <c r="E44" s="11" t="n">
-        <v>-18.5</v>
+        <v>-23</v>
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t>خصم تكلفة شحنة مرتجعة - طلب #767 (مزامنة إدارية)</t>
+          <t>إصدار بوليصات لعدد 1 طلب - أرامكس (Treek)</t>
         </is>
       </c>
       <c r="G44" s="10" t="n"/>
@@ -43928,11 +45706,11 @@
     <row r="45" ht="24" customHeight="1">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>#1379</t>
+          <t>#1407</t>
         </is>
       </c>
       <c r="B45" s="27" t="n">
-        <v>41816.74444444444</v>
+        <v>42547.88958333333</v>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
@@ -43941,7 +45719,7 @@
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>admin_deduction</t>
+          <t>شحن</t>
         </is>
       </c>
       <c r="E45" s="11" t="n">
@@ -43949,7 +45727,7 @@
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t>خصم تكلفة شحنة مرتجعة - طلب #1376 (مزامنة إدارية)</t>
+          <t>إصدار بوليصات لعدد 1 طلب - SMSA - سمسا (عبر نظام الشحنات)</t>
         </is>
       </c>
       <c r="G45" s="10" t="n"/>
@@ -43962,28 +45740,28 @@
     <row r="46" ht="24" customHeight="1">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>#1378</t>
+          <t>#1406</t>
         </is>
       </c>
       <c r="B46" s="27" t="n">
-        <v>41816.74236111111</v>
+        <v>42547.87777777778</v>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>مؤسسة اواني القيصرية التجارية</t>
+          <t>عبدالرحمن المطيري</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>إيداع</t>
+          <t>شحن</t>
         </is>
       </c>
       <c r="E46" s="11" t="n">
-        <v>18.5</v>
+        <v>-141</v>
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t>شحن إداري للرصيد - تعويض عن شحنة - بواسطة المدير #1</t>
+          <t>إصدار بوليصات لعدد 6 طلب - SMSA - سمسا (عبر نظام الشحنات)</t>
         </is>
       </c>
       <c r="G46" s="10" t="n"/>
@@ -43996,32 +45774,474 @@
     <row r="47" ht="24" customHeight="1">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>#1368</t>
+          <t>#1405</t>
         </is>
       </c>
       <c r="B47" s="27" t="n">
-        <v>41816.58055555556</v>
+        <v>42547.83541666667</v>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>احمد محمد بن عبدالله الرزق</t>
+          <t>ليد إكسبرس</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>إيداع</t>
+          <t>استرداد</t>
         </is>
       </c>
       <c r="E47" s="11" t="n">
-        <v>500</v>
+        <v>23.5</v>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>شحن رصيد عبر تحويل بنكي - مرجع: 151_1781434588_b102d0cd.jpeg [صورة: 151_1781434588_b102d0cd.jpeg]</t>
+          <t>استرداد تكلفة شحن - إلغاء طلب #2062</t>
         </is>
       </c>
       <c r="G47" s="10" t="n"/>
       <c r="H47" s="10" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="24" customHeight="1">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>#1404</t>
+        </is>
+      </c>
+      <c r="B48" s="27" t="n">
+        <v>42547.83541666667</v>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>ليد إكسبرس</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>شحن</t>
+        </is>
+      </c>
+      <c r="E48" s="11" t="n">
+        <v>-23.5</v>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>إصدار بوليصات لعدد 1 طلب - SMSA - سمسا (عبر نظام الشحنات)</t>
+        </is>
+      </c>
+      <c r="G48" s="10" t="n"/>
+      <c r="H48" s="10" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="24" customHeight="1">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>#1403</t>
+        </is>
+      </c>
+      <c r="B49" s="27" t="n">
+        <v>42547.83472222222</v>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>ليد إكسبرس</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>استرداد</t>
+        </is>
+      </c>
+      <c r="E49" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>استرداد تكلفة شحن - إلغاء طلب #2061</t>
+        </is>
+      </c>
+      <c r="G49" s="10" t="n"/>
+      <c r="H49" s="10" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="24" customHeight="1">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>#1402</t>
+        </is>
+      </c>
+      <c r="B50" s="27" t="n">
+        <v>42547.83472222222</v>
+      </c>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>ليد إكسبرس</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>شحن</t>
+        </is>
+      </c>
+      <c r="E50" s="11" t="n">
+        <v>-20</v>
+      </c>
+      <c r="F50" s="10" t="inlineStr">
+        <is>
+          <t>إصدار بوليصات لعدد 1 طلب - aramex ( استلام من الفرع ) (عبر نظام الشحنات)</t>
+        </is>
+      </c>
+      <c r="G50" s="10" t="n"/>
+      <c r="H50" s="10" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="24" customHeight="1">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>#1401</t>
+        </is>
+      </c>
+      <c r="B51" s="27" t="n">
+        <v>42547.79305555556</v>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>فهد احمد</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>شحن</t>
+        </is>
+      </c>
+      <c r="E51" s="11" t="n">
+        <v>-20</v>
+      </c>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>إصدار بوليصات لعدد 1 طلب - aramex ( استلام من الفرع ) (عبر نظام الشحنات)</t>
+        </is>
+      </c>
+      <c r="G51" s="10" t="n"/>
+      <c r="H51" s="10" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="24" customHeight="1">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>#1400</t>
+        </is>
+      </c>
+      <c r="B52" s="27" t="n">
+        <v>42547.78680555556</v>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>فارس احمد</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>إيداع</t>
+        </is>
+      </c>
+      <c r="E52" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
+          <t>شحن رصيد عبر تحويل بنكي - مرجع: 132_1781625226_c8bee3fa.jpeg [صورة: 132_1781625226_c8bee3fa.jpeg]</t>
+        </is>
+      </c>
+      <c r="G52" s="10" t="n"/>
+      <c r="H52" s="10" t="inlineStr">
+        <is>
+          <t>البنك</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="24" customHeight="1">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>#1399</t>
+        </is>
+      </c>
+      <c r="B53" s="27" t="n">
+        <v>42547.77638888889</v>
+      </c>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>احمد محمد بن عبدالله الرزق</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>شحن</t>
+        </is>
+      </c>
+      <c r="E53" s="11" t="n">
+        <v>-117.5</v>
+      </c>
+      <c r="F53" s="10" t="inlineStr">
+        <is>
+          <t>إصدار بوليصات لعدد 5 طلب - SMSA - سمسا (عبر نظام الشحنات)</t>
+        </is>
+      </c>
+      <c r="G53" s="10" t="n"/>
+      <c r="H53" s="10" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="24" customHeight="1">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>#1398</t>
+        </is>
+      </c>
+      <c r="B54" s="27" t="n">
+        <v>42547.64375</v>
+      </c>
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>مؤسسة اواني القيصرية التجارية</t>
+        </is>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>شحن</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="n">
+        <v>-18.5</v>
+      </c>
+      <c r="F54" s="10" t="inlineStr">
+        <is>
+          <t>إصدار بوليصات لعدد 1 طلب - SMSA - سمسا (عبر نظام الشحنات)</t>
+        </is>
+      </c>
+      <c r="G54" s="10" t="n"/>
+      <c r="H54" s="10" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="24" customHeight="1">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>#1397</t>
+        </is>
+      </c>
+      <c r="B55" s="27" t="n">
+        <v>42547.13611111111</v>
+      </c>
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>نوف مرزوق العتيبي</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>إيداع</t>
+        </is>
+      </c>
+      <c r="E55" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="F55" s="10" t="inlineStr">
+        <is>
+          <t>شحن رصيد عبر تحويل بنكي - مرجع: 88_1781569012_9e0ddea1.png [صورة: 88_1781569012_9e0ddea1.png]</t>
+        </is>
+      </c>
+      <c r="G55" s="10" t="n"/>
+      <c r="H55" s="10" t="inlineStr">
+        <is>
+          <t>البنك</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="24" customHeight="1">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>#1382</t>
+        </is>
+      </c>
+      <c r="B56" s="27" t="n">
+        <v>41816.91944444444</v>
+      </c>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>فارس احمد</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>إيداع</t>
+        </is>
+      </c>
+      <c r="E56" s="11" t="n">
+        <v>252</v>
+      </c>
+      <c r="F56" s="10" t="inlineStr">
+        <is>
+          <t>شحن رصيد عبر تحويل بنكي - مرجع: 132_1781463851_d66934a2.jpeg [صورة: 132_1781463851_d66934a2.jpeg]</t>
+        </is>
+      </c>
+      <c r="G56" s="10" t="n"/>
+      <c r="H56" s="10" t="inlineStr">
+        <is>
+          <t>البنك</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="24" customHeight="1">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>#1380</t>
+        </is>
+      </c>
+      <c r="B57" s="27" t="n">
+        <v>41816.74444444444</v>
+      </c>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>مؤسسة اواني القيصرية التجارية</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>admin_deduction</t>
+        </is>
+      </c>
+      <c r="E57" s="11" t="n">
+        <v>-18.5</v>
+      </c>
+      <c r="F57" s="10" t="inlineStr">
+        <is>
+          <t>خصم تكلفة شحنة مرتجعة - طلب #767 (مزامنة إدارية)</t>
+        </is>
+      </c>
+      <c r="G57" s="10" t="n"/>
+      <c r="H57" s="10" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="24" customHeight="1">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>#1379</t>
+        </is>
+      </c>
+      <c r="B58" s="27" t="n">
+        <v>41816.74444444444</v>
+      </c>
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>عبدالرحمن المطيري</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>admin_deduction</t>
+        </is>
+      </c>
+      <c r="E58" s="11" t="n">
+        <v>-23.5</v>
+      </c>
+      <c r="F58" s="10" t="inlineStr">
+        <is>
+          <t>خصم تكلفة شحنة مرتجعة - طلب #1376 (مزامنة إدارية)</t>
+        </is>
+      </c>
+      <c r="G58" s="10" t="n"/>
+      <c r="H58" s="10" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="24" customHeight="1">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>#1378</t>
+        </is>
+      </c>
+      <c r="B59" s="27" t="n">
+        <v>41816.74236111111</v>
+      </c>
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>مؤسسة اواني القيصرية التجارية</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>إيداع</t>
+        </is>
+      </c>
+      <c r="E59" s="11" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F59" s="10" t="inlineStr">
+        <is>
+          <t>شحن إداري للرصيد - تعويض عن شحنة - بواسطة المدير #1</t>
+        </is>
+      </c>
+      <c r="G59" s="10" t="n"/>
+      <c r="H59" s="10" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="24" customHeight="1">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>#1368</t>
+        </is>
+      </c>
+      <c r="B60" s="27" t="n">
+        <v>41816.58055555556</v>
+      </c>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>احمد محمد بن عبدالله الرزق</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>إيداع</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="n">
+        <v>500</v>
+      </c>
+      <c r="F60" s="10" t="inlineStr">
+        <is>
+          <t>شحن رصيد عبر تحويل بنكي - مرجع: 151_1781434588_b102d0cd.jpeg [صورة: 151_1781434588_b102d0cd.jpeg]</t>
+        </is>
+      </c>
+      <c r="G60" s="10" t="n"/>
+      <c r="H60" s="10" t="inlineStr">
         <is>
           <t>البنك</t>
         </is>

</xml_diff>

<commit_message>
Add remote sync and raw ingestion
</commit_message>
<xml_diff>
--- a/output/lead6_report.xlsx
+++ b/output/lead6_report.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخصات" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تفاصيل شهر 6" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الاسعار" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="العمليات المالية" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كشف الحساب" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ملخصات" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="تفاصيل شهر 6" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="الاسعار" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="العمليات المالية" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="كشف الحساب" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'تفاصيل شهر 6'!$A$1:$X$476</definedName>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>1241.06</v>
+        <v>1241.059999999995</v>
       </c>
       <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="n"/>
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>1253.31</v>
+        <v>1253.309999999995</v>
       </c>
       <c r="C14" s="4" t="n"/>
       <c r="D14" s="4" t="n"/>
@@ -45520,21 +45520,21 @@
         </is>
       </c>
       <c r="Q478" s="7" t="n">
-        <v>9118.77</v>
+        <v>9118.770000000044</v>
       </c>
       <c r="R478" s="7" t="n">
-        <v>7825.73</v>
+        <v>7825.729999999912</v>
       </c>
       <c r="S478" s="15" t="n"/>
       <c r="T478" s="7" t="n">
-        <v>1241.06</v>
+        <v>1241.059999999995</v>
       </c>
       <c r="U478" s="7" t="n">
         <v>4.25</v>
       </c>
       <c r="V478" s="15" t="n"/>
       <c r="W478" s="7" t="n">
-        <v>1253.31</v>
+        <v>1253.309999999995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>